<commit_message>
Update TSTT_Board_Data.xlsx with latest data
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tsttcott-my.sharepoint.com/personal/csimeon_tstt_co_tt/Documents/Financial Analysis/TSTT_Board_Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="6_{31AE12F9-1F43-4E41-A874-E34D2BA7A817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7175AD98-0455-4599-AA52-7CC3D00F064E}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="6_{31AE12F9-1F43-4E41-A874-E34D2BA7A817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFC64BF6-6740-4EE9-93AB-0D21FC1ACBA4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Summary" sheetId="1" r:id="rId1"/>
@@ -620,6 +620,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -746,11 +749,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -780,8 +784,15 @@
     <xf numFmtId="9" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -1049,7 +1060,7 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="22" customWidth="1"/>
-    <col min="4" max="6" width="14" customWidth="1"/>
+    <col min="4" max="6" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
   </cols>
@@ -1090,14 +1101,14 @@
       <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2">
-        <v>1580</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1520</v>
-      </c>
-      <c r="F2" s="4">
-        <v>1490</v>
+      <c r="D2" s="12">
+        <v>219588802.66</v>
+      </c>
+      <c r="E2" s="12">
+        <v>189588802.66</v>
+      </c>
+      <c r="F2" s="12">
+        <v>220788802.66</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>177</v>
@@ -1116,14 +1127,14 @@
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3">
-        <v>445</v>
-      </c>
-      <c r="E3" s="3">
-        <v>460</v>
-      </c>
-      <c r="F3" s="5">
-        <v>420</v>
+      <c r="D3" s="12">
+        <v>97157262.870000005</v>
+      </c>
+      <c r="E3" s="12">
+        <v>67157262.870000005</v>
+      </c>
+      <c r="F3" s="12">
+        <v>98357262.870000005</v>
       </c>
       <c r="G3" s="9" t="s">
         <v>181</v>
@@ -1142,14 +1153,14 @@
       <c r="C4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="2">
-        <v>185</v>
-      </c>
-      <c r="E4" s="2">
-        <v>195</v>
-      </c>
-      <c r="F4" s="4">
-        <v>170</v>
+      <c r="D4" s="12">
+        <v>6054943.790000014</v>
+      </c>
+      <c r="E4" s="12">
+        <v>-23945056.209999986</v>
+      </c>
+      <c r="F4" s="12">
+        <v>7254943.790000014</v>
       </c>
       <c r="G4" s="9" t="s">
         <v>181</v>
@@ -1168,14 +1179,17 @@
       <c r="C5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3">
-        <v>28.2</v>
-      </c>
-      <c r="E5" s="3">
-        <v>30.2</v>
-      </c>
-      <c r="F5" s="5">
-        <v>28.2</v>
+      <c r="D5" s="11">
+        <f>D3/D2</f>
+        <v>0.4424508977374102</v>
+      </c>
+      <c r="E5" s="11">
+        <f t="shared" ref="E5:F5" si="0">E3/E2</f>
+        <v>0.35422589270969135</v>
+      </c>
+      <c r="F5" s="11">
+        <f t="shared" si="0"/>
+        <v>0.44548120957684445</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>181</v>
@@ -1195,13 +1209,13 @@
         <v>16</v>
       </c>
       <c r="D6" s="2">
-        <v>265</v>
+        <v>265000000</v>
       </c>
       <c r="E6" s="2">
-        <v>220</v>
+        <v>22000000</v>
       </c>
       <c r="F6" s="4">
-        <v>217</v>
+        <v>217111111</v>
       </c>
       <c r="G6" s="9" t="s">
         <v>177</v>
@@ -3682,27 +3696,21 @@
         <v>0.39418982145184989</v>
       </c>
       <c r="F2" s="2">
-        <f>B2-30000000</f>
         <v>135461792.16999999</v>
       </c>
       <c r="G2" s="2">
-        <f>C2-30000000</f>
         <v>35223354.31259539</v>
       </c>
       <c r="H2" s="2">
-        <f>D2-30000000</f>
         <v>-23722087.487404615</v>
       </c>
       <c r="I2" s="2">
-        <f>B2+1200000</f>
         <v>166661792.16999999</v>
       </c>
       <c r="J2" s="2">
-        <f t="shared" ref="J2:K11" si="0">C2+1200000</f>
         <v>66423354.31259539</v>
       </c>
       <c r="K2" s="2">
-        <f t="shared" si="0"/>
         <v>7477912.5125953853</v>
       </c>
     </row>
@@ -3720,31 +3728,25 @@
         <v>29629601.979999982</v>
       </c>
       <c r="E3" s="10">
-        <f t="shared" ref="E3:E11" si="1">C3/B3</f>
+        <f t="shared" ref="E3:E11" si="0">C3/B3</f>
         <v>0.45237021375698966</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:H11" si="2">B3-30000000</f>
         <v>138114139.21000001</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" si="2"/>
         <v>46049829.090000018</v>
       </c>
       <c r="H3" s="2">
-        <f t="shared" si="2"/>
         <v>-370398.02000001818</v>
       </c>
       <c r="I3" s="2">
-        <f t="shared" ref="I3:I11" si="3">B3+1200000</f>
         <v>169314139.21000001</v>
       </c>
       <c r="J3" s="2">
-        <f t="shared" si="0"/>
         <v>77249829.090000018</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" si="0"/>
         <v>30829601.979999982</v>
       </c>
     </row>
@@ -3762,31 +3764,25 @@
         <v>-5433120.2799999937</v>
       </c>
       <c r="E4" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.25110230522271276</v>
       </c>
       <c r="F4" s="2">
-        <f t="shared" si="2"/>
         <v>135003060.18000001</v>
       </c>
       <c r="G4" s="2">
-        <f t="shared" si="2"/>
         <v>11432648.780000001</v>
       </c>
       <c r="H4" s="2">
-        <f t="shared" si="2"/>
         <v>-35433120.279999994</v>
       </c>
       <c r="I4" s="2">
-        <f t="shared" si="3"/>
         <v>166203060.18000001</v>
       </c>
       <c r="J4" s="2">
-        <f t="shared" si="0"/>
         <v>42632648.780000001</v>
       </c>
       <c r="K4" s="2">
-        <f t="shared" si="0"/>
         <v>-4233120.2799999937</v>
       </c>
     </row>
@@ -3804,31 +3800,25 @@
         <v>25240036.869999968</v>
       </c>
       <c r="E5" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.47245018082821755</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" si="2"/>
         <v>134228182.28999996</v>
       </c>
       <c r="G5" s="2">
-        <f t="shared" si="2"/>
         <v>47589634.419999957</v>
       </c>
       <c r="H5" s="2">
-        <f t="shared" si="2"/>
         <v>-4759963.1300000325</v>
       </c>
       <c r="I5" s="2">
-        <f t="shared" si="3"/>
         <v>165428182.28999996</v>
       </c>
       <c r="J5" s="2">
-        <f t="shared" si="0"/>
         <v>78789634.419999957</v>
       </c>
       <c r="K5" s="2">
-        <f t="shared" si="0"/>
         <v>26440036.869999968</v>
       </c>
     </row>
@@ -3846,31 +3836,25 @@
         <v>2452908.3699999452</v>
       </c>
       <c r="E6" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.26733176918587631</v>
       </c>
       <c r="F6" s="2">
-        <f t="shared" si="2"/>
         <v>132138200.08000001</v>
       </c>
       <c r="G6" s="2">
-        <f t="shared" si="2"/>
         <v>13344691.879999995</v>
       </c>
       <c r="H6" s="2">
-        <f t="shared" si="2"/>
         <v>-27547091.630000055</v>
       </c>
       <c r="I6" s="2">
-        <f t="shared" si="3"/>
         <v>163338200.08000001</v>
       </c>
       <c r="J6" s="2">
-        <f t="shared" si="0"/>
         <v>44544691.879999995</v>
       </c>
       <c r="K6" s="2">
-        <f t="shared" si="0"/>
         <v>3652908.3699999452</v>
       </c>
     </row>
@@ -3888,31 +3872,25 @@
         <v>-3851804.6799999699</v>
       </c>
       <c r="E7" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.25303400495945899</v>
       </c>
       <c r="F7" s="2">
-        <f t="shared" si="2"/>
         <v>193865976.34999999</v>
       </c>
       <c r="G7" s="2">
-        <f t="shared" si="2"/>
         <v>26645704.570000023</v>
       </c>
       <c r="H7" s="2">
-        <f t="shared" si="2"/>
         <v>-33851804.67999997</v>
       </c>
       <c r="I7" s="2">
-        <f t="shared" si="3"/>
         <v>225065976.34999999</v>
       </c>
       <c r="J7" s="2">
-        <f t="shared" si="0"/>
         <v>57845704.570000023</v>
       </c>
       <c r="K7" s="2">
-        <f t="shared" si="0"/>
         <v>-2651804.6799999699</v>
       </c>
     </row>
@@ -3930,31 +3908,25 @@
         <v>30509086.749999985</v>
       </c>
       <c r="E8" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.35941145088720255</v>
       </c>
       <c r="F8" s="2">
-        <f t="shared" si="2"/>
         <v>159426200.56189248</v>
       </c>
       <c r="G8" s="2">
-        <f t="shared" si="2"/>
         <v>38081945.579999998</v>
       </c>
       <c r="H8" s="2">
-        <f t="shared" si="2"/>
         <v>509086.7499999851</v>
       </c>
       <c r="I8" s="2">
-        <f t="shared" si="3"/>
         <v>190626200.56189248</v>
       </c>
       <c r="J8" s="2">
-        <f t="shared" si="0"/>
         <v>69281945.579999998</v>
       </c>
       <c r="K8" s="2">
-        <f t="shared" si="0"/>
         <v>31709086.749999985</v>
       </c>
     </row>
@@ -3972,31 +3944,25 @@
         <v>15814747.380000003</v>
       </c>
       <c r="E9" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.29826415219544128</v>
       </c>
       <c r="F9" s="2">
-        <f t="shared" si="2"/>
         <v>186028154.09</v>
       </c>
       <c r="G9" s="2">
-        <f t="shared" si="2"/>
         <v>34433454.229999997</v>
       </c>
       <c r="H9" s="2">
-        <f t="shared" si="2"/>
         <v>-14185252.619999997</v>
       </c>
       <c r="I9" s="2">
-        <f t="shared" si="3"/>
         <v>217228154.09</v>
       </c>
       <c r="J9" s="2">
-        <f t="shared" si="0"/>
         <v>65633454.229999997</v>
       </c>
       <c r="K9" s="2">
-        <f t="shared" si="0"/>
         <v>17014747.380000003</v>
       </c>
     </row>
@@ -4014,31 +3980,25 @@
         <v>6054943.790000014</v>
       </c>
       <c r="E10" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.4424508977374102</v>
       </c>
       <c r="F10" s="2">
-        <f t="shared" si="2"/>
         <v>189588802.66</v>
       </c>
       <c r="G10" s="2">
-        <f t="shared" si="2"/>
         <v>67157262.870000005</v>
       </c>
       <c r="H10" s="2">
-        <f t="shared" si="2"/>
         <v>-23945056.209999986</v>
       </c>
       <c r="I10" s="2">
-        <f t="shared" si="3"/>
         <v>220788802.66</v>
       </c>
       <c r="J10" s="2">
-        <f t="shared" si="0"/>
         <v>98357262.870000005</v>
       </c>
       <c r="K10" s="2">
-        <f t="shared" si="0"/>
         <v>7254943.790000014</v>
       </c>
     </row>
@@ -4056,31 +4016,25 @@
         <v>6054943.790000014</v>
       </c>
       <c r="E11" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.4424508977374102</v>
       </c>
       <c r="F11" s="2">
-        <f t="shared" si="2"/>
         <v>189588802.66</v>
       </c>
       <c r="G11" s="2">
-        <f t="shared" si="2"/>
         <v>67157262.870000005</v>
       </c>
       <c r="H11" s="2">
-        <f t="shared" si="2"/>
         <v>-23945056.209999986</v>
       </c>
       <c r="I11" s="2">
-        <f t="shared" si="3"/>
         <v>220788802.66</v>
       </c>
       <c r="J11" s="2">
-        <f t="shared" si="0"/>
         <v>98357262.870000005</v>
       </c>
       <c r="K11" s="2">
-        <f t="shared" si="0"/>
         <v>7254943.790000014</v>
       </c>
     </row>
@@ -8401,18 +8355,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8434,6 +8388,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46063F7-F7F9-4CDE-8387-57A2670C9E1C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F30D9A8-DF0C-4BE8-8230-FB1B79303CAC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -8447,12 +8409,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46063F7-F7F9-4CDE-8387-57A2670C9E1C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add real subscriber data to Consumer Sales (Prepaid, Postpaid, WTTx)
- Load subscriber_base_apw.xlsx (monthly_pivot sheet) in build_board_data.py
- Populate Subscribers and compute ARPU = Revenue / Subscribers for the three
  mobile segments; TV / Residential Security / Other remain at 0 (no source data)
- Compute YoY_Change_Pct for CUR_FY ACT months from prior-year actuals
- Fix avg_arpu metric card in Consumer page: was Revenue(TT$M)*Subs (wrong units),
  now ARPU*Subs weighted average in TT$
- Regenerate TSTT_Board_Data.xlsx with populated subscriber metrics

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -6398,13 +6398,13 @@
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>418249</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>82.56398303402997</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -6426,13 +6426,13 @@
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>104426</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>298.7116873192501</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -6454,13 +6454,13 @@
       </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>103490</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>159.3746960092762</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -6566,13 +6566,13 @@
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>408145</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>78.27391123252765</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -6594,13 +6594,13 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>105314</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>306.3371519456104</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -6622,13 +6622,13 @@
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>104166</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>158.1244472284623</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -6734,13 +6734,13 @@
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>406256</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>80.13345489051241</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -6762,13 +6762,13 @@
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>105051</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>312.3410083673643</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -6790,13 +6790,13 @@
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>103778</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>158.349268727476</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -6902,13 +6902,13 @@
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>415715</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>0</v>
+        <v>78.16455357636845</v>
       </c>
       <c r="H20" t="n">
         <v>0</v>
@@ -6930,13 +6930,13 @@
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>104606</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>303.8614050819265</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -6958,13 +6958,13 @@
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>104939</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>157.5617372949999</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -7070,13 +7070,13 @@
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>0</v>
+        <v>408999</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>0</v>
+        <v>80.63161526067303</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -7098,13 +7098,13 @@
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>0</v>
+        <v>104695</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>301.6925609627968</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -7126,13 +7126,13 @@
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>105189</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>157.2668884579186</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -7238,13 +7238,13 @@
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>402155</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>0</v>
+        <v>79.02668214991735</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -7266,13 +7266,13 @@
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>104853</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>302.3931534624664</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -7294,13 +7294,13 @@
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>104516</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>156.7259296184316</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -7406,13 +7406,13 @@
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>405228</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>82.14163665886859</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -7434,13 +7434,13 @@
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
-        <v>0</v>
+        <v>105409</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>299.2338304129628</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -7462,13 +7462,13 @@
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>105018</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>155.0814416576206</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -7574,13 +7574,13 @@
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>398400</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>79.1263904116466</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -7602,13 +7602,13 @@
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>105592</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>300.1656039283279</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -7630,13 +7630,13 @@
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>104708</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>157.536751633113</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -7742,13 +7742,13 @@
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>407702</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>82.53160364678122</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -7770,13 +7770,13 @@
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
-        <v>0</v>
+        <v>107204</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>296.2280401850677</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>
@@ -7798,13 +7798,13 @@
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
-        <v>0</v>
+        <v>105134</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>157.9829472863203</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
@@ -7910,13 +7910,13 @@
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>401325</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>0</v>
+        <v>79.60490936273594</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
@@ -7938,13 +7938,13 @@
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
-        <v>0</v>
+        <v>107374</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>0</v>
+        <v>297.3199102203512</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
@@ -7966,13 +7966,13 @@
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>0</v>
+        <v>103936</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>158.2723479833744</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -8078,13 +8078,13 @@
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
-        <v>0</v>
+        <v>393549</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>0</v>
+        <v>77.26434598995297</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
@@ -8106,13 +8106,13 @@
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
-        <v>0</v>
+        <v>106525</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>0</v>
+        <v>300.5152455292185</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
@@ -8134,13 +8134,13 @@
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>102974</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>0</v>
+        <v>153.1831536115913</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
@@ -8246,13 +8246,13 @@
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
-        <v>0</v>
+        <v>399776</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>0</v>
+        <v>80.13519651004563</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -8274,13 +8274,13 @@
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
-        <v>0</v>
+        <v>106046</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>0</v>
+        <v>296.2934243630123</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
@@ -8302,13 +8302,13 @@
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
-        <v>0</v>
+        <v>102423</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>158.6333118537828</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -8446,13 +8446,13 @@
         <v>31354854</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>107275</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>290.7785286413425</v>
       </c>
       <c r="H75" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update financial_data source; fold new DATA and Voice lines into Consumer Other
- Replace financial_data.xlsx with updated version (adds DATA and Voice
  descriptions under Consumer Sales BU, +74 rows)
- Add DATA and Voice to the Other segment bucket in build_consumer_sales
  so they are captured in totals without adding new segments to the page
- Regenerate TSTT_Board_Data.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -6534,7 +6534,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-689804.02</v>
+        <v>-642839.04</v>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
@@ -6702,7 +6702,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>536694.5699999999</v>
+        <v>681794.1399999999</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
@@ -6870,7 +6870,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>491066.8599999999</v>
+        <v>608367.9699999999</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -7038,7 +7038,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2180470.21</v>
+        <v>2339715.25</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
@@ -7206,7 +7206,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1099723.64</v>
+        <v>1173605.93</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
@@ -7374,7 +7374,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1195406.27</v>
+        <v>1243125.76</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
@@ -7542,7 +7542,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>287703.76</v>
+        <v>318455.0599999999</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>-203220.0600000001</v>
+        <v>-142458.1900000001</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
@@ -7878,7 +7878,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>482209.2</v>
+        <v>550175.77</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
@@ -8046,7 +8046,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>-239327.8100000001</v>
+        <v>-128753.3900000001</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
@@ -8214,7 +8214,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>25281.7899999998</v>
+        <v>-56792.2100000002</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
@@ -8382,7 +8382,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>20410778.79</v>
+        <v>20370819.67</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
@@ -8472,7 +8472,9 @@
       <c r="C76" t="n">
         <v>16493687.29</v>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="n">
+        <v>12408697.21022757</v>
+      </c>
       <c r="E76" t="n">
         <v>0</v>
       </c>
@@ -8530,7 +8532,9 @@
       <c r="C78" t="n">
         <v>1282307.83</v>
       </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="D78" t="n">
+        <v>1560782.257073873</v>
+      </c>
       <c r="E78" t="n">
         <v>0</v>
       </c>
@@ -8556,10 +8560,10 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-689804.02</v>
+        <v>-642839.04</v>
       </c>
       <c r="D79" t="n">
-        <v>-521275.871928572</v>
+        <v>-513435.1648404523</v>
       </c>
       <c r="E79" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Populate Amplia Commercial tab from Amplia KPI file
- Add AMP_KPI_SRC constant and _amp_metric() helper to parse the
  wide-pivot Amplia KPI spreadsheet by metric label + FY row label
- Add build_amplia_commercial() to extract ARPU, Gross Adds vs Budget,
  and Churn vs Budget for FY25/26 Actual (Apr-25 through Feb-26)
- Move SUBS_SRC constant to module level alongside other source constants
- AMPLIA_Commercial now has 11 real rows (was 0); Tab 2 will render

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -1888,7 +1888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1941,6 +1941,402 @@
         <is>
           <t>Sales_Target</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Apr-25</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>363.7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1792</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1605</v>
+      </c>
+      <c r="E2" t="n">
+        <v>911</v>
+      </c>
+      <c r="F2" t="n">
+        <v>708</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1792</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>May-25</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>367.21</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1853</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1605</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1209</v>
+      </c>
+      <c r="F3" t="n">
+        <v>713</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1853</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jun-25</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>370.37</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1591</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1702</v>
+      </c>
+      <c r="E4" t="n">
+        <v>737</v>
+      </c>
+      <c r="F4" t="n">
+        <v>718</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1591</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1702</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jul-25</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>368.66</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1959</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1732</v>
+      </c>
+      <c r="E5" t="n">
+        <v>863</v>
+      </c>
+      <c r="F5" t="n">
+        <v>725</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>1959</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1732</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aug-25</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>363.48</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1985</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1869</v>
+      </c>
+      <c r="E6" t="n">
+        <v>782</v>
+      </c>
+      <c r="F6" t="n">
+        <v>731</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1985</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sep-25</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>353.3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1775</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1744</v>
+      </c>
+      <c r="E7" t="n">
+        <v>893</v>
+      </c>
+      <c r="F7" t="n">
+        <v>739</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1775</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1744</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oct-25</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>370.57</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1624</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1615</v>
+      </c>
+      <c r="E8" t="n">
+        <v>772</v>
+      </c>
+      <c r="F8" t="n">
+        <v>772</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>1624</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>364.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1662</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1853</v>
+      </c>
+      <c r="E9" t="n">
+        <v>847</v>
+      </c>
+      <c r="F9" t="n">
+        <v>850</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>1662</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dec-25</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>349.58</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1899</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1955</v>
+      </c>
+      <c r="E10" t="n">
+        <v>681</v>
+      </c>
+      <c r="F10" t="n">
+        <v>850</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1899</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1955</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>358.18</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1998</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1738</v>
+      </c>
+      <c r="E11" t="n">
+        <v>512</v>
+      </c>
+      <c r="F11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1998</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>348.56</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1927</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1605</v>
+      </c>
+      <c r="E12" t="n">
+        <v>771</v>
+      </c>
+      <c r="F12" t="n">
+        <v>900</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1927</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add P&L Breakdown tab and fix 9-column financial_data.xlsx schema
- Fix column rename in main() to handle new Sub-category column (9 cols)
- Update Business Sales segment map with recategorised descriptions
- Add build_pnl_breakdown() for consolidated Revenue/COS/OPEX/EBITDA cascade
- Scale PnL_Breakdown sheet in data_loader.py
- Add "P&L Breakdown" as first tab on Financial Performance page with
  stacked bar revenue by group, COS by group, cascade trend line, and
  latest-month waterfall (Rev → COS → GP → OPEX → EBITDA)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -19,6 +19,7 @@
     <sheet name="DPDI" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="AMPLIA_Financial" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="AMPLIA_Commercial" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="PnL_Breakdown" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2344,6 +2345,1350 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_Rev</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_COS</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_COS_AOP</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_Rev</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_COS</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_COS_AOP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_Rev</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_COS</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_COS_AOP</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_Rev</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_COS</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_COS_AOP</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_Rev</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_COS</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_COS_AOP</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Rev</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Total_COS</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Total_COS_AOP</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Total_OPEX</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Total_OPEX_AOP</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA_AOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Apr-25</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>91096868.77000003</v>
+      </c>
+      <c r="C2" t="n">
+        <v>91861724.33722802</v>
+      </c>
+      <c r="D2" t="n">
+        <v>14010859.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14694559</v>
+      </c>
+      <c r="F2" t="n">
+        <v>46030788.94</v>
+      </c>
+      <c r="G2" t="n">
+        <v>46038101.31160618</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2993618.490000005</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3914465.000221079</v>
+      </c>
+      <c r="J2" t="n">
+        <v>25447329.81</v>
+      </c>
+      <c r="K2" t="n">
+        <v>25306707</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5052508.66</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5424966.671355191</v>
+      </c>
+      <c r="N2" t="n">
+        <v>938594.01</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-2699339.957355191</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-1834298</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-2173327.611799635</v>
+      </c>
+      <c r="V2" t="n">
+        <v>161513581.53</v>
+      </c>
+      <c r="W2" t="n">
+        <v>161455631.371479</v>
+      </c>
+      <c r="X2" t="n">
+        <v>20440369.03</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>22095623.50577664</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>70534458.91</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>79142846.41900846</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>70625668.58000004</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>60277161.4466939</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>May-25</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>90216607.98999998</v>
+      </c>
+      <c r="C3" t="n">
+        <v>94477769.34541556</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14495304.21</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17949064</v>
+      </c>
+      <c r="F3" t="n">
+        <v>49130568.39000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>46867653.30865601</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3677532.320000003</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3957438.122569739</v>
+      </c>
+      <c r="J3" t="n">
+        <v>26113220.11</v>
+      </c>
+      <c r="K3" t="n">
+        <v>25695738</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4772772.48</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5536017.290862304</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1487994.94</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>567680.38</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-2760275.319999993</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-1925581.206862304</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-2007753</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-2193497.231306748</v>
+      </c>
+      <c r="V3" t="n">
+        <v>164188116.11</v>
+      </c>
+      <c r="W3" t="n">
+        <v>166064018.1272093</v>
+      </c>
+      <c r="X3" t="n">
+        <v>21505536.39</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>25483982.6281253</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>75810568.88496403</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>80294802.45533194</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>66878419.69503598</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>60345233.04375206</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Jun-25</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>92076140.39</v>
+      </c>
+      <c r="C4" t="n">
+        <v>95355430.26794931</v>
+      </c>
+      <c r="D4" t="n">
+        <v>14320378.37</v>
+      </c>
+      <c r="E4" t="n">
+        <v>17149115</v>
+      </c>
+      <c r="F4" t="n">
+        <v>47973222.28</v>
+      </c>
+      <c r="G4" t="n">
+        <v>49271362.95392575</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4074876.499999999</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5669547.26212224</v>
+      </c>
+      <c r="J4" t="n">
+        <v>26264263.11999999</v>
+      </c>
+      <c r="K4" t="n">
+        <v>26117859</v>
+      </c>
+      <c r="L4" t="n">
+        <v>4868498.779999999</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5667066.271218739</v>
+      </c>
+      <c r="N4" t="n">
+        <v>849467.6</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-2099197.270000011</v>
+      </c>
+      <c r="S4" t="n">
+        <v>-1873232.94721874</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-2506000</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-2213383.211663184</v>
+      </c>
+      <c r="V4" t="n">
+        <v>165063896.12</v>
+      </c>
+      <c r="W4" t="n">
+        <v>169808297.9546563</v>
+      </c>
+      <c r="X4" t="n">
+        <v>20975434.03</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>26499213.7676778</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>61139026.484</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>85830882.96297152</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>82957229.07600001</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>57538201.22400703</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Jul-25</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>92352581.47000001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>93050892.72757138</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12750826.02</v>
+      </c>
+      <c r="E5" t="n">
+        <v>14026249</v>
+      </c>
+      <c r="F5" t="n">
+        <v>47587833.92</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57191021.8726786</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4168335.999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9034393.60408327</v>
+      </c>
+      <c r="J5" t="n">
+        <v>26813033.17</v>
+      </c>
+      <c r="K5" t="n">
+        <v>26548290</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4888500.08</v>
+      </c>
+      <c r="M5" t="n">
+        <v>5903059.725788871</v>
+      </c>
+      <c r="N5" t="n">
+        <v>811866.53</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-2103522.920000017</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-1884423.78178887</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-1959028</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-2231587.666233315</v>
+      </c>
+      <c r="V5" t="n">
+        <v>165461792.17</v>
+      </c>
+      <c r="W5" t="n">
+        <v>175868411.7184611</v>
+      </c>
+      <c r="X5" t="n">
+        <v>20043009.1</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>26946489.66363882</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>69348866.35740462</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>80665674.77810179</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>77217920.58259538</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>68316247.27672051</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aug-25</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>91710972.35000001</v>
+      </c>
+      <c r="C6" t="n">
+        <v>94922246.92634216</v>
+      </c>
+      <c r="D6" t="n">
+        <v>14354491.13</v>
+      </c>
+      <c r="E6" t="n">
+        <v>14258018</v>
+      </c>
+      <c r="F6" t="n">
+        <v>50292629.49</v>
+      </c>
+      <c r="G6" t="n">
+        <v>48659101.64179683</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6465935.41</v>
+      </c>
+      <c r="I6" t="n">
+        <v>12013341.36505904</v>
+      </c>
+      <c r="J6" t="n">
+        <v>26736564.21</v>
+      </c>
+      <c r="K6" t="n">
+        <v>27145842</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4838473.97</v>
+      </c>
+      <c r="M6" t="n">
+        <v>6177159.525720645</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1175208.19</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-1801235.030000001</v>
+      </c>
+      <c r="S6" t="n">
+        <v>-1913793.101720645</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-1992385</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-2252756.46616509</v>
+      </c>
+      <c r="V6" t="n">
+        <v>168114139.21</v>
+      </c>
+      <c r="W6" t="n">
+        <v>169776028.3664184</v>
+      </c>
+      <c r="X6" t="n">
+        <v>23860890.50999999</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>30410137.4246146</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>57139294.3366566</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>79676394.27091196</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>87175279.61334342</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>59749496.67089179</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sep-25</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>90128359.70000002</v>
+      </c>
+      <c r="C7" t="n">
+        <v>95256419.87762924</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12401311.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14335147</v>
+      </c>
+      <c r="F7" t="n">
+        <v>49694116.7</v>
+      </c>
+      <c r="G7" t="n">
+        <v>55726352.92198627</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3994895.449999998</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10118915.56281924</v>
+      </c>
+      <c r="J7" t="n">
+        <v>26178595.18</v>
+      </c>
+      <c r="K7" t="n">
+        <v>27695774</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4184827.09</v>
+      </c>
+      <c r="M7" t="n">
+        <v>6376459.743183928</v>
+      </c>
+      <c r="N7" t="n">
+        <v>931282.51</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-1929293.910000026</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-1922257.799183928</v>
+      </c>
+      <c r="T7" t="n">
+        <v>3383837.23</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-2269421.683628372</v>
+      </c>
+      <c r="V7" t="n">
+        <v>165003060.18</v>
+      </c>
+      <c r="W7" t="n">
+        <v>177718919.9004316</v>
+      </c>
+      <c r="X7" t="n">
+        <v>24159246.57</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>28775475.6223748</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>88389572.78</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>82771329.67812991</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>53343312.77000001</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>66232114.59992689</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oct-25</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>90463809.88</v>
+      </c>
+      <c r="C8" t="n">
+        <v>98674774.79495525</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12708159.02</v>
+      </c>
+      <c r="E8" t="n">
+        <v>21300316</v>
+      </c>
+      <c r="F8" t="n">
+        <v>47588262.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>50227856.88656416</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3634572.31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4313561.95097963</v>
+      </c>
+      <c r="J8" t="n">
+        <v>27643427.7</v>
+      </c>
+      <c r="K8" t="n">
+        <v>28012879</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4731653.62</v>
+      </c>
+      <c r="M8" t="n">
+        <v>6614449.37043488</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1079682.51</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-2547000</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-1940573.426434881</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-2298255</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-2287737.310879325</v>
+      </c>
+      <c r="V8" t="n">
+        <v>164228182.29</v>
+      </c>
+      <c r="W8" t="n">
+        <v>176668068.1550846</v>
+      </c>
+      <c r="X8" t="n">
+        <v>18970504.95</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>30382465.01053519</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>57673660.21000001</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>79397077.23208006</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>87917309.37999997</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>66948525.91246931</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>88902786.52</v>
+      </c>
+      <c r="C9" t="n">
+        <v>101914509.4918081</v>
+      </c>
+      <c r="D9" t="n">
+        <v>14703578.64</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20616008</v>
+      </c>
+      <c r="F9" t="n">
+        <v>46360935.73</v>
+      </c>
+      <c r="G9" t="n">
+        <v>62508806.64368133</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3859427.17</v>
+      </c>
+      <c r="I9" t="n">
+        <v>15348644.75734568</v>
+      </c>
+      <c r="J9" t="n">
+        <v>27356236.08</v>
+      </c>
+      <c r="K9" t="n">
+        <v>28597259</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4885687.32</v>
+      </c>
+      <c r="M9" t="n">
+        <v>6872938.37913241</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2157709.42</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1265375</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-2639467.669999987</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-1960946.43513241</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-2476148</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-2308110.319576854</v>
+      </c>
+      <c r="V9" t="n">
+        <v>162138200.08</v>
+      </c>
+      <c r="W9" t="n">
+        <v>192827759.600357</v>
+      </c>
+      <c r="X9" t="n">
+        <v>22237920.13</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>40971355.81690125</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>83238334.97</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>86895985.01353751</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>55622267.49000001</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>65020418.76991829</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dec-25</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>92056924.37999998</v>
+      </c>
+      <c r="C10" t="n">
+        <v>105112539.7619839</v>
+      </c>
+      <c r="D10" t="n">
+        <v>13669721.21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>24118315</v>
+      </c>
+      <c r="F10" t="n">
+        <v>53126006.13</v>
+      </c>
+      <c r="G10" t="n">
+        <v>64564850.52355281</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9149765.82</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8733145.425684026</v>
+      </c>
+      <c r="J10" t="n">
+        <v>26941579.35</v>
+      </c>
+      <c r="K10" t="n">
+        <v>28975873</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5015843.060000001</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7145591.801489527</v>
+      </c>
+      <c r="N10" t="n">
+        <v>53778662.25</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>45087125</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-2037195.75999999</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-1983866.857489527</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-2653712</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-2331030.741933972</v>
+      </c>
+      <c r="V10" t="n">
+        <v>223865976.35</v>
+      </c>
+      <c r="W10" t="n">
+        <v>198731718.3280472</v>
+      </c>
+      <c r="X10" t="n">
+        <v>70268743.09</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>38137896.48523958</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>85821328.38999999</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>87502690.83408965</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>67899678.31999999</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>73151131.00871794</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>89570651.43000001</v>
+      </c>
+      <c r="C11" t="n">
+        <v>94892293.2192031</v>
+      </c>
+      <c r="D11" t="n">
+        <v>12704569.97</v>
+      </c>
+      <c r="E11" t="n">
+        <v>14100869.41</v>
+      </c>
+      <c r="F11" t="n">
+        <v>45833455.48</v>
+      </c>
+      <c r="G11" t="n">
+        <v>55775449.37978129</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5159112.889999998</v>
+      </c>
+      <c r="I11" t="n">
+        <v>8740611.206033947</v>
+      </c>
+      <c r="J11" t="n">
+        <v>26995058.56189249</v>
+      </c>
+      <c r="K11" t="n">
+        <v>29393218</v>
+      </c>
+      <c r="L11" t="n">
+        <v>5063916.859999999</v>
+      </c>
+      <c r="M11" t="n">
+        <v>7317661.119463768</v>
+      </c>
+      <c r="N11" t="n">
+        <v>29378388.9</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>24393875</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-2351353.810000002</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-1996431.175463768</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-2773000</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-2343595.059908213</v>
+      </c>
+      <c r="V11" t="n">
+        <v>189426200.5618925</v>
+      </c>
+      <c r="W11" t="n">
+        <v>181170857.5901873</v>
+      </c>
+      <c r="X11" t="n">
+        <v>44548474.72</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>28955637.27558951</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>65462556.84424999</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>81283075.27646777</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>79538114.5476425</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>70992145.03813002</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>86627198.53</v>
+      </c>
+      <c r="C12" t="n">
+        <v>96008362.93721315</v>
+      </c>
+      <c r="D12" t="n">
+        <v>12420253.18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>18468843.41</v>
+      </c>
+      <c r="F12" t="n">
+        <v>49594614.91</v>
+      </c>
+      <c r="G12" t="n">
+        <v>52209344.05719531</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4697652.45</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3764030.682719573</v>
+      </c>
+      <c r="J12" t="n">
+        <v>27244862.09</v>
+      </c>
+      <c r="K12" t="n">
+        <v>29880629</v>
+      </c>
+      <c r="L12" t="n">
+        <v>10988379.38</v>
+      </c>
+      <c r="M12" t="n">
+        <v>7495389.334991091</v>
+      </c>
+      <c r="N12" t="n">
+        <v>53371865.19</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>44301206.73</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-810386.6299999952</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-2004757.390991091</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-905000</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-2351921.275435536</v>
+      </c>
+      <c r="V12" t="n">
+        <v>216028154.09</v>
+      </c>
+      <c r="W12" t="n">
+        <v>179252406.770084</v>
+      </c>
+      <c r="X12" t="n">
+        <v>71502491.73999999</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>28516432.75227513</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>66132145.10608834</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>81717722.67198595</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>78514328.51391169</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>69078251.34582293</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>108214511.69</v>
+      </c>
+      <c r="C13" t="n">
+        <v>94631079.54768565</v>
+      </c>
+      <c r="D13" t="n">
+        <v>13045142.61</v>
+      </c>
+      <c r="E13" t="n">
+        <v>17868311</v>
+      </c>
+      <c r="F13" t="n">
+        <v>82925659.89</v>
+      </c>
+      <c r="G13" t="n">
+        <v>66884533.84582798</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1836751.030000004</v>
+      </c>
+      <c r="I13" t="n">
+        <v>14313238.62119834</v>
+      </c>
+      <c r="J13" t="n">
+        <v>29642976.66</v>
+      </c>
+      <c r="K13" t="n">
+        <v>30155964</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4603785.73</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7734181.205156771</v>
+      </c>
+      <c r="N13" t="n">
+        <v>908753.9300000001</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>243119.99</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-2103099.51000002</v>
+      </c>
+      <c r="S13" t="n">
+        <v>-2985901.491156771</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-14457484.17</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-2365427.145601215</v>
+      </c>
+      <c r="V13" t="n">
+        <v>219588802.66</v>
+      </c>
+      <c r="W13" t="n">
+        <v>199291615.1690235</v>
+      </c>
+      <c r="X13" t="n">
+        <v>5271315.190000005</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>40490394.2807539</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>111963280.11</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>86293632.73162086</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>107853458.94</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>72567588.15664874</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>91096868.77000003</v>
+      </c>
+      <c r="C14" t="n">
+        <v>80274532.4636035</v>
+      </c>
+      <c r="D14" t="n">
+        <v>14010859.5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>10442347.08371727</v>
+      </c>
+      <c r="F14" t="n">
+        <v>46030788.94</v>
+      </c>
+      <c r="G14" t="n">
+        <v>46530148.5645342</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2993618.490000005</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3881417.21134247</v>
+      </c>
+      <c r="J14" t="n">
+        <v>25447329.81</v>
+      </c>
+      <c r="K14" t="n">
+        <v>28894159.2091278</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5052508.66</v>
+      </c>
+      <c r="M14" t="n">
+        <v>5142998.307669034</v>
+      </c>
+      <c r="N14" t="n">
+        <v>938594.01</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-2953301.1165</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-1834298</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-2217682.8665</v>
+      </c>
+      <c r="V14" t="n">
+        <v>161513581.53</v>
+      </c>
+      <c r="W14" t="n">
+        <v>153681628.0207655</v>
+      </c>
+      <c r="X14" t="n">
+        <v>20440369.03</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>17464854.98622877</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>70534458.91</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>78962885.94843617</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>70625668.58000004</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>57308900.91610059</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -9140,7 +10485,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20926355.99</v>
+        <v>21600881.77</v>
       </c>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
@@ -9171,9 +10516,7 @@
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -9198,13 +10541,13 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>-2388946.55</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -9357,7 +10700,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>21692749.5</v>
+        <v>23516584.79</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
@@ -9388,9 +10731,7 @@
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -9415,13 +10756,13 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>70522.28999999905</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>0</v>
       </c>
@@ -9574,7 +10915,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>21491993.13</v>
+        <v>24672867.84</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
@@ -9605,9 +10946,7 @@
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="n">
-        <v>0</v>
-      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>0</v>
       </c>
@@ -9632,13 +10971,13 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>-2171392.18</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>0</v>
       </c>
@@ -9791,7 +11130,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>21825311.91</v>
+        <v>22784846.65</v>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
@@ -9822,9 +11161,7 @@
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
-      <c r="D27" t="n">
-        <v>0</v>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>0</v>
       </c>
@@ -9849,13 +11186,13 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>-25886.26999999955</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>0</v>
       </c>
@@ -10008,7 +11345,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>21055288.57</v>
+        <v>24421045.17</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
@@ -10039,9 +11376,7 @@
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
-      <c r="D34" t="n">
-        <v>0</v>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>0</v>
       </c>
@@ -10066,13 +11401,13 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>436868.2199999997</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0</v>
       </c>
@@ -10225,7 +11560,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>21345475.79</v>
+        <v>25308730.56</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
@@ -10256,9 +11591,7 @@
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
-      <c r="D41" t="n">
-        <v>0</v>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -10283,13 +11616,13 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>717630.66</v>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -10442,7 +11775,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>21573947.98</v>
+        <v>25128771.74000001</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
@@ -10473,9 +11806,7 @@
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
-      <c r="D48" t="n">
-        <v>0</v>
-      </c>
+      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0</v>
       </c>
@@ -10500,13 +11831,13 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>-1799860.500000001</v>
+      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0</v>
       </c>
@@ -10659,7 +11990,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>22191200.33</v>
+        <v>24094943.07</v>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
@@ -10690,9 +12021,7 @@
         </is>
       </c>
       <c r="C55" t="inlineStr"/>
-      <c r="D55" t="n">
-        <v>0</v>
-      </c>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0</v>
       </c>
@@ -10717,13 +12046,13 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>-2180681.55</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>0</v>
       </c>
@@ -10876,7 +12205,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>21147362.27</v>
+        <v>27525526.53</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
@@ -10907,9 +12236,7 @@
         </is>
       </c>
       <c r="C62" t="inlineStr"/>
-      <c r="D62" t="n">
-        <v>0</v>
-      </c>
+      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>0</v>
       </c>
@@ -10934,13 +12261,13 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-      <c r="D63" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>-2501556.88</v>
+      </c>
+      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>0</v>
       </c>
@@ -11093,7 +12420,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>20442625.87</v>
+        <v>22235459.22</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
@@ -11124,9 +12451,7 @@
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
-      <c r="D69" t="n">
-        <v>0</v>
-      </c>
+      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>0</v>
       </c>
@@ -11151,13 +12476,13 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>-1754001.68</v>
+      </c>
+      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>0</v>
       </c>
@@ -11310,7 +12635,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>21501364.72</v>
+        <v>26971656.22</v>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
@@ -11341,9 +12666,7 @@
         </is>
       </c>
       <c r="C76" t="inlineStr"/>
-      <c r="D76" t="n">
-        <v>0</v>
-      </c>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>0</v>
       </c>
@@ -11368,13 +12691,13 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>-1027449.279999998</v>
+      </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>0</v>
       </c>
@@ -11527,7 +12850,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>20402030.17</v>
+        <v>23740185.99</v>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
@@ -11558,9 +12881,7 @@
         </is>
       </c>
       <c r="C83" t="inlineStr"/>
-      <c r="D83" t="n">
-        <v>0</v>
-      </c>
+      <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
         <v>0</v>
       </c>
@@ -11585,13 +12906,13 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr"/>
-      <c r="D84" t="n">
-        <v>0</v>
-      </c>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>29994897.77</v>
+      </c>
+      <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
         <v>0</v>
       </c>
@@ -11750,10 +13071,10 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>20926355.99</v>
+        <v>21600881.77</v>
       </c>
       <c r="D89" t="n">
-        <v>21848000.15291695</v>
+        <v>23191742.98291694</v>
       </c>
       <c r="E89" t="n">
         <v>0</v>
@@ -11784,7 +13105,7 @@
       </c>
       <c r="C90" t="inlineStr"/>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>3755696.517725</v>
       </c>
       <c r="E90" t="n">
         <v>0</v>
@@ -11810,12 +13131,14 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Managed</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr"/>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>-2388946.55</v>
+      </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>-170396.3628571429</v>
       </c>
       <c r="E91" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add Enterprise Scorecard page with 2x2 balanced-scorecard layout
Populate KPI_Summary sheet with 17 KPIs across four sections:
- Financial (6): Revenue, EBITDA, PAT, EBITDA Margin, FCF, CAPEX/Revenue
- Customer (4): NPS, Postpaid Churn, Complaints, Fibre Net-Adds
- Network (3): Network Availability, MTTR, Install Lead Time
- People (4): Engagement Score, Women in Leadership, Voluntary Attrition,
  Critical Vacancy Fill

Page features:
- Custom header with period derived dynamically from KPI data
- 2x2 quadrant grid with section-specific accent colours
- RAG dot from Status field + direction arrow coloured by whether
  the direction is favourable (higher-is-better vs lower-is-better sets)
- Within-2%-of-AOP check renders neutral amber arrow
- CONFIDENTIAL footer

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,6 +647,474 @@
         </is>
       </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Free Cash Flow</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>42912000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TT$M</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CAPEX/Revenue</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>32</v>
+      </c>
+      <c r="E8" t="n">
+        <v>35</v>
+      </c>
+      <c r="F8" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>pts</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Postpaid Churn</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Complaints</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Fibre Net-Adds</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F11" t="n">
+        <v>900</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>subs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Network Availability</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MTTR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>🟢</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>hrs</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Network</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Install Lead Time</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Engagement Score</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>68</v>
+      </c>
+      <c r="E15" t="n">
+        <v>72</v>
+      </c>
+      <c r="F15" t="n">
+        <v>65</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Women in Leadership</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Voluntary Attrition</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.092</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>🔴</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Critical Vacancy Fill</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>🟡</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>%</t>
         </is>

</xml_diff>

<commit_message>
Add FY2027 OPEX plan from AOP file; restore Apr-26 actuals
Loads OPEX_AOP_FY2027.xlsx and aggregates by category and month to
populate Plan values for the full FY2027 year (Apr-26 to Mar-27,
TT$1,258M total). Includes load_fy2027_opex.py loader script with
actuals-preservation logic. Apr-26 actuals recovered from git history
after initial load inadvertently zeroed them out.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -90,12 +90,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -1900,6 +1899,17 @@
   </sheetPr>
   <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="7.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="12.140625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="4.42578125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="5.7109375" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="12" bestFit="1" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2364,6 +2374,17 @@
   </sheetPr>
   <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="15.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="20.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="15" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="9" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="8.28515625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="12.140625" bestFit="1" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4168,7 +4189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" bestFit="1" customWidth="1" min="2" max="4"/>
@@ -4176,7 +4197,6 @@
     <col width="13.85546875" bestFit="1" customWidth="1" min="6" max="6"/>
     <col width="12.140625" bestFit="1" customWidth="1" min="7" max="7"/>
     <col width="12.7109375" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="12" bestFit="1" customWidth="1" min="9" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4220,21 +4240,6 @@
           <t>PAT_AOP</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Revenue_LY</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>EBITDA_LY</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>PAT_LY</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4598,15 +4603,6 @@
       </c>
       <c r="H14" t="n">
         <v>-26733913.62156836</v>
-      </c>
-      <c r="I14" t="n">
-        <v>161513581.53</v>
-      </c>
-      <c r="J14" t="n">
-        <v>70625668.58000004</v>
-      </c>
-      <c r="K14" t="n">
-        <v>14592872.86000008</v>
       </c>
     </row>
   </sheetData>
@@ -4622,6 +4618,12 @@
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="9" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4742,11 +4744,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4755,38 +4757,38 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Variance</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Variance_Pct</t>
         </is>
       </c>
     </row>
-    <row r="2" hidden="1">
+    <row r="2">
       <c r="A2" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4810,7 +4812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" hidden="1">
+    <row r="3">
       <c r="A3" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4834,7 +4836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" hidden="1">
+    <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4858,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" hidden="1">
+    <row r="5">
       <c r="A5" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4879,7 +4881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" hidden="1">
+    <row r="6">
       <c r="A6" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4903,7 +4905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" hidden="1">
+    <row r="7">
       <c r="A7" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4927,7 +4929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" hidden="1">
+    <row r="8">
       <c r="A8" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4951,7 +4953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" hidden="1">
+    <row r="9">
       <c r="A9" t="inlineStr">
         <is>
           <t>Apr-25</t>
@@ -4975,7 +4977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" hidden="1">
+    <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -4999,7 +5001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" hidden="1">
+    <row r="11">
       <c r="A11" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5023,7 +5025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" hidden="1">
+    <row r="12">
       <c r="A12" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5047,7 +5049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" hidden="1">
+    <row r="13">
       <c r="A13" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5068,7 +5070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" hidden="1">
+    <row r="14">
       <c r="A14" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5092,7 +5094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" hidden="1">
+    <row r="15">
       <c r="A15" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5116,7 +5118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" hidden="1">
+    <row r="16">
       <c r="A16" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5140,7 +5142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" hidden="1">
+    <row r="17">
       <c r="A17" t="inlineStr">
         <is>
           <t>May-25</t>
@@ -5164,7 +5166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" hidden="1">
+    <row r="18">
       <c r="A18" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5188,7 +5190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" hidden="1">
+    <row r="19">
       <c r="A19" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5212,7 +5214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" hidden="1">
+    <row r="20">
       <c r="A20" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5236,7 +5238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" hidden="1">
+    <row r="21">
       <c r="A21" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5257,7 +5259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" hidden="1">
+    <row r="22">
       <c r="A22" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5281,7 +5283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" hidden="1">
+    <row r="23">
       <c r="A23" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5305,7 +5307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" hidden="1">
+    <row r="24">
       <c r="A24" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5329,7 +5331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" hidden="1">
+    <row r="25">
       <c r="A25" t="inlineStr">
         <is>
           <t>Jun-25</t>
@@ -5353,7 +5355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" hidden="1">
+    <row r="26">
       <c r="A26" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5364,7 +5366,7 @@
           <t>Advertising &amp; PR.</t>
         </is>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" t="n">
         <v>1493909.770000001</v>
       </c>
       <c r="D26" t="n">
@@ -5377,7 +5379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" hidden="1">
+    <row r="27">
       <c r="A27" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5388,7 +5390,7 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" t="n">
         <v>2770972</v>
       </c>
       <c r="D27" t="n">
@@ -5401,7 +5403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" hidden="1">
+    <row r="28">
       <c r="A28" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5412,7 +5414,7 @@
           <t>Consultancy &amp; Other Fees.</t>
         </is>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" t="n">
         <v>2740749.29</v>
       </c>
       <c r="D28" t="n">
@@ -5425,7 +5427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" hidden="1">
+    <row r="29">
       <c r="A29" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5436,7 +5438,6 @@
           <t>DIG. PROD DEV &amp; INNOV</t>
         </is>
       </c>
-      <c r="C29" s="3" t="n"/>
       <c r="D29" t="n">
         <v>962630.9</v>
       </c>
@@ -5447,7 +5448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" hidden="1">
+    <row r="30">
       <c r="A30" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5458,7 +5459,7 @@
           <t>Maintenance.</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" t="n">
         <v>18958609.92</v>
       </c>
       <c r="D30" t="n">
@@ -5471,7 +5472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" hidden="1">
+    <row r="31">
       <c r="A31" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5482,7 +5483,7 @@
           <t>Other Operating Expenses.</t>
         </is>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" t="n">
         <v>18038804.21</v>
       </c>
       <c r="D31" t="n">
@@ -5495,7 +5496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" hidden="1">
+    <row r="32">
       <c r="A32" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5506,7 +5507,7 @@
           <t>Personnel.</t>
         </is>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" t="n">
         <v>20186695.95740462</v>
       </c>
       <c r="D32" t="n">
@@ -5519,7 +5520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" hidden="1">
+    <row r="33">
       <c r="A33" t="inlineStr">
         <is>
           <t>Jul-25</t>
@@ -5530,7 +5531,7 @@
           <t>Professional.</t>
         </is>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" t="n">
         <v>5159125.21</v>
       </c>
       <c r="D33" t="n">
@@ -5543,7 +5544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" hidden="1">
+    <row r="34">
       <c r="A34" t="inlineStr">
         <is>
           <t>Aug-25</t>
@@ -5825,7 +5826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" hidden="1">
+    <row r="46">
       <c r="A46" t="inlineStr">
         <is>
           <t>Sep-25</t>
@@ -5849,7 +5850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" hidden="1">
+    <row r="47">
       <c r="A47" t="inlineStr">
         <is>
           <t>Sep-25</t>
@@ -5873,7 +5874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" hidden="1">
+    <row r="48">
       <c r="A48" t="inlineStr">
         <is>
           <t>Sep-25</t>
@@ -5897,7 +5898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" hidden="1">
+    <row r="49">
       <c r="A49" t="inlineStr">
         <is>
           <t>Sep-25</t>
@@ -5921,7 +5922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" hidden="1">
+    <row r="50">
       <c r="A50" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -5945,7 +5946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" hidden="1">
+    <row r="51">
       <c r="A51" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -5969,7 +5970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" hidden="1">
+    <row r="52">
       <c r="A52" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -5993,7 +5994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" hidden="1">
+    <row r="53">
       <c r="A53" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -6014,7 +6015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" hidden="1">
+    <row r="54">
       <c r="A54" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -6038,7 +6039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" hidden="1">
+    <row r="55">
       <c r="A55" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -6062,7 +6063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" hidden="1">
+    <row r="56">
       <c r="A56" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -6086,7 +6087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" hidden="1">
+    <row r="57">
       <c r="A57" t="inlineStr">
         <is>
           <t>Oct-25</t>
@@ -6110,7 +6111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" hidden="1">
+    <row r="58">
       <c r="A58" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6134,7 +6135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" hidden="1">
+    <row r="59">
       <c r="A59" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6158,7 +6159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" hidden="1">
+    <row r="60">
       <c r="A60" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6182,7 +6183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" hidden="1">
+    <row r="61">
       <c r="A61" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6203,7 +6204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" hidden="1">
+    <row r="62">
       <c r="A62" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6227,7 +6228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" hidden="1">
+    <row r="63">
       <c r="A63" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6251,7 +6252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" hidden="1">
+    <row r="64">
       <c r="A64" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6275,7 +6276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" hidden="1">
+    <row r="65">
       <c r="A65" t="inlineStr">
         <is>
           <t>Nov-25</t>
@@ -6299,7 +6300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" hidden="1">
+    <row r="66">
       <c r="A66" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6323,7 +6324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" hidden="1">
+    <row r="67">
       <c r="A67" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6347,7 +6348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" hidden="1">
+    <row r="68">
       <c r="A68" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6371,7 +6372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" hidden="1">
+    <row r="69">
       <c r="A69" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6392,7 +6393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" hidden="1">
+    <row r="70">
       <c r="A70" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6416,7 +6417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" hidden="1">
+    <row r="71">
       <c r="A71" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6440,7 +6441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" hidden="1">
+    <row r="72">
       <c r="A72" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6464,7 +6465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" hidden="1">
+    <row r="73">
       <c r="A73" t="inlineStr">
         <is>
           <t>Dec-25</t>
@@ -6488,7 +6489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" hidden="1">
+    <row r="74">
       <c r="A74" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6512,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" hidden="1">
+    <row r="75">
       <c r="A75" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6536,7 +6537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" hidden="1">
+    <row r="76">
       <c r="A76" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6560,7 +6561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" hidden="1">
+    <row r="77">
       <c r="A77" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6581,7 +6582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" hidden="1">
+    <row r="78">
       <c r="A78" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6605,7 +6606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" hidden="1">
+    <row r="79">
       <c r="A79" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6629,7 +6630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" hidden="1">
+    <row r="80">
       <c r="A80" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6653,7 +6654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" hidden="1">
+    <row r="81">
       <c r="A81" t="inlineStr">
         <is>
           <t>Jan-26</t>
@@ -6677,7 +6678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" hidden="1">
+    <row r="82">
       <c r="A82" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6701,7 +6702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" hidden="1">
+    <row r="83">
       <c r="A83" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6725,7 +6726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" hidden="1">
+    <row r="84">
       <c r="A84" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6749,7 +6750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" hidden="1">
+    <row r="85">
       <c r="A85" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6770,7 +6771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" hidden="1">
+    <row r="86">
       <c r="A86" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6794,7 +6795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" hidden="1">
+    <row r="87">
       <c r="A87" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6818,7 +6819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" hidden="1">
+    <row r="88">
       <c r="A88" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6842,7 +6843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" hidden="1">
+    <row r="89">
       <c r="A89" t="inlineStr">
         <is>
           <t>Feb-26</t>
@@ -6866,7 +6867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" hidden="1">
+    <row r="90">
       <c r="A90" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -6890,7 +6891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" hidden="1">
+    <row r="91">
       <c r="A91" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -6914,7 +6915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" hidden="1">
+    <row r="92">
       <c r="A92" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -6938,7 +6939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" hidden="1">
+    <row r="93">
       <c r="A93" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -6959,7 +6960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" hidden="1">
+    <row r="94">
       <c r="A94" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -6983,7 +6984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" hidden="1">
+    <row r="95">
       <c r="A95" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -7007,7 +7008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" hidden="1">
+    <row r="96">
       <c r="A96" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -7031,7 +7032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" hidden="1">
+    <row r="97">
       <c r="A97" t="inlineStr">
         <is>
           <t>Mar-26</t>
@@ -7055,7 +7056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" hidden="1">
+    <row r="98">
       <c r="A98" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7063,23 +7064,23 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Advertising &amp; PR.</t>
+          <t>Advertising &amp; PR</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2968556.690000001</v>
+        <v>2968556.69</v>
       </c>
       <c r="D98" t="n">
         <v>2248453.405862648</v>
       </c>
       <c r="E98" t="n">
-        <v>0</v>
+        <v>-2248453.405862648</v>
       </c>
       <c r="F98" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="99">
       <c r="A99" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7094,16 +7095,16 @@
         <v>2558987.34</v>
       </c>
       <c r="D99" t="n">
-        <v>3641316.303154886</v>
+        <v>3641316.303154887</v>
       </c>
       <c r="E99" t="n">
-        <v>0</v>
+        <v>-3641316.303154887</v>
       </c>
       <c r="F99" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="100">
       <c r="A100" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7111,23 +7112,23 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Consultancy &amp; Other Fees.</t>
+          <t>Consultancy &amp; Other Fees</t>
         </is>
       </c>
       <c r="C100" t="n">
         <v>3475330.73</v>
       </c>
       <c r="D100" t="n">
-        <v>4825993.819165427</v>
+        <v>4717492.952380952</v>
       </c>
       <c r="E100" t="n">
-        <v>0</v>
+        <v>-4717492.952380952</v>
       </c>
       <c r="F100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="101">
       <c r="A101" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7135,17 +7136,23 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>DIG. PROD DEV &amp; INNOV</t>
-        </is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>22798838.08</v>
+      </c>
+      <c r="D101" t="n">
+        <v>22845189.22992514</v>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
+        <v>-22845189.22992514</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="102">
       <c r="A102" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7153,23 +7160,23 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Maintenance.</t>
+          <t>Other Operating Expenses</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>22798838.08</v>
+        <v>15329485.2</v>
       </c>
       <c r="D102" t="n">
-        <v>23065367.61818174</v>
+        <v>17641296.31599329</v>
       </c>
       <c r="E102" t="n">
-        <v>0</v>
+        <v>-17641296.31599329</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="103">
       <c r="A103" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7177,23 +7184,23 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Other Operating Expenses.</t>
+          <t>Personnel</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>15329485.2</v>
+        <v>19177303.91</v>
       </c>
       <c r="D103" t="n">
-        <v>17265858.47323616</v>
+        <v>22430669.71354279</v>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
+        <v>-22430669.71354279</v>
       </c>
       <c r="F103" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="104">
       <c r="A104" t="inlineStr">
         <is>
           <t>Apr-26</t>
@@ -7201,93 +7208,1872 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Personnel.</t>
+          <t>Professional</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>19177303.91</v>
+        <v>4225956.96</v>
       </c>
       <c r="D104" t="n">
-        <v>21277967.28114248</v>
+        <v>9258148.492380952</v>
       </c>
       <c r="E104" t="n">
-        <v>0</v>
+        <v>-9258148.492380952</v>
       </c>
       <c r="F104" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" hidden="1">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Apr-26</t>
+          <t>May-26</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Professional.</t>
+          <t>Advertising &amp; PR</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4225956.96</v>
+        <v>0</v>
       </c>
       <c r="D105" t="n">
-        <v>6637929.047692832</v>
+        <v>3241953.232895536</v>
       </c>
       <c r="E105" t="n">
-        <v>0</v>
+        <v>-3241953.232895536</v>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" hidden="1"/>
-    <row r="107" hidden="1"/>
-    <row r="108" hidden="1"/>
-    <row r="109" hidden="1"/>
-    <row r="110" hidden="1"/>
-    <row r="111" hidden="1"/>
-    <row r="112" hidden="1"/>
-    <row r="113" hidden="1"/>
-    <row r="114" hidden="1"/>
-    <row r="115" hidden="1"/>
-    <row r="116" hidden="1"/>
-    <row r="117" hidden="1"/>
-    <row r="118" hidden="1"/>
-    <row r="119" hidden="1"/>
-    <row r="120" hidden="1"/>
-    <row r="121" hidden="1"/>
-    <row r="122" hidden="1"/>
-    <row r="123" hidden="1"/>
-    <row r="124" hidden="1"/>
-    <row r="125" hidden="1"/>
-    <row r="126" hidden="1"/>
-    <row r="127" hidden="1"/>
-    <row r="128" hidden="1"/>
-    <row r="129" hidden="1"/>
-    <row r="130" hidden="1"/>
-    <row r="131" hidden="1"/>
-    <row r="132" hidden="1"/>
-    <row r="133" hidden="1"/>
-    <row r="134" hidden="1"/>
-    <row r="135" hidden="1"/>
-    <row r="136" hidden="1"/>
-    <row r="137" hidden="1"/>
-    <row r="138" hidden="1"/>
-    <row r="139" hidden="1"/>
-    <row r="140" hidden="1"/>
-    <row r="141" hidden="1"/>
-    <row r="142" hidden="1"/>
-    <row r="143" hidden="1"/>
-    <row r="144" hidden="1"/>
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" t="n">
+        <v>3168047.030440447</v>
+      </c>
+      <c r="E106" t="n">
+        <v>-3168047.030440447</v>
+      </c>
+      <c r="F106" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" t="n">
+        <v>4905665.142857144</v>
+      </c>
+      <c r="E107" t="n">
+        <v>-4905665.142857144</v>
+      </c>
+      <c r="F107" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>0</v>
+      </c>
+      <c r="D108" t="n">
+        <v>23147297.86274611</v>
+      </c>
+      <c r="E108" t="n">
+        <v>-23147297.86274611</v>
+      </c>
+      <c r="F108" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>0</v>
+      </c>
+      <c r="D109" t="n">
+        <v>17646306.05536446</v>
+      </c>
+      <c r="E109" t="n">
+        <v>-17646306.05536446</v>
+      </c>
+      <c r="F109" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" t="n">
+        <v>22591612.33270326</v>
+      </c>
+      <c r="E110" t="n">
+        <v>-22591612.33270326</v>
+      </c>
+      <c r="F110" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" t="n">
+        <v>9426348.492380952</v>
+      </c>
+      <c r="E111" t="n">
+        <v>-9426348.492380952</v>
+      </c>
+      <c r="F111" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>0</v>
+      </c>
+      <c r="D112" t="n">
+        <v>5201350.327907625</v>
+      </c>
+      <c r="E112" t="n">
+        <v>-5201350.327907625</v>
+      </c>
+      <c r="F112" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D113" t="n">
+        <v>3294321.145640145</v>
+      </c>
+      <c r="E113" t="n">
+        <v>-3294321.145640145</v>
+      </c>
+      <c r="F113" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D114" t="n">
+        <v>5082945.212857143</v>
+      </c>
+      <c r="E114" t="n">
+        <v>-5082945.212857143</v>
+      </c>
+      <c r="F114" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" t="n">
+        <v>23871463.00056273</v>
+      </c>
+      <c r="E115" t="n">
+        <v>-23871463.00056273</v>
+      </c>
+      <c r="F115" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" t="n">
+        <v>19474521.73444509</v>
+      </c>
+      <c r="E116" t="n">
+        <v>-19474521.73444509</v>
+      </c>
+      <c r="F116" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" t="n">
+        <v>22522911.54131892</v>
+      </c>
+      <c r="E117" t="n">
+        <v>-22522911.54131892</v>
+      </c>
+      <c r="F117" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Jun-26</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>0</v>
+      </c>
+      <c r="D118" t="n">
+        <v>12090103.49238095</v>
+      </c>
+      <c r="E118" t="n">
+        <v>-12090103.49238095</v>
+      </c>
+      <c r="F118" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" t="n">
+        <v>2842128.722017645</v>
+      </c>
+      <c r="E119" t="n">
+        <v>-2842128.722017645</v>
+      </c>
+      <c r="F119" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>0</v>
+      </c>
+      <c r="D120" t="n">
+        <v>3725840.471526688</v>
+      </c>
+      <c r="E120" t="n">
+        <v>-3725840.471526688</v>
+      </c>
+      <c r="F120" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" t="n">
+        <v>5040297.142857144</v>
+      </c>
+      <c r="E121" t="n">
+        <v>-5040297.142857144</v>
+      </c>
+      <c r="F121" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>0</v>
+      </c>
+      <c r="D122" t="n">
+        <v>22771503.68704942</v>
+      </c>
+      <c r="E122" t="n">
+        <v>-22771503.68704942</v>
+      </c>
+      <c r="F122" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" t="n">
+        <v>110707370.9709836</v>
+      </c>
+      <c r="E123" t="n">
+        <v>-110707370.9709836</v>
+      </c>
+      <c r="F123" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" t="n">
+        <v>22657637.09599318</v>
+      </c>
+      <c r="E124" t="n">
+        <v>-22657637.09599318</v>
+      </c>
+      <c r="F124" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" t="n">
+        <v>10129315.49238095</v>
+      </c>
+      <c r="E125" t="n">
+        <v>-10129315.49238095</v>
+      </c>
+      <c r="F125" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" t="n">
+        <v>4722333.82309229</v>
+      </c>
+      <c r="E126" t="n">
+        <v>-4722333.82309229</v>
+      </c>
+      <c r="F126" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" t="n">
+        <v>3794023.364505047</v>
+      </c>
+      <c r="E127" t="n">
+        <v>-3794023.364505047</v>
+      </c>
+      <c r="F127" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>0</v>
+      </c>
+      <c r="D128" t="n">
+        <v>4217492.952380952</v>
+      </c>
+      <c r="E128" t="n">
+        <v>-4217492.952380952</v>
+      </c>
+      <c r="F128" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" t="n">
+        <v>23101642.49688293</v>
+      </c>
+      <c r="E129" t="n">
+        <v>-23101642.49688293</v>
+      </c>
+      <c r="F129" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" t="n">
+        <v>18031437.18467504</v>
+      </c>
+      <c r="E130" t="n">
+        <v>-18031437.18467504</v>
+      </c>
+      <c r="F130" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" t="n">
+        <v>22986653.2146912</v>
+      </c>
+      <c r="E131" t="n">
+        <v>-22986653.2146912</v>
+      </c>
+      <c r="F131" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Aug-26</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" t="n">
+        <v>9875546.492380952</v>
+      </c>
+      <c r="E132" t="n">
+        <v>-9875546.492380952</v>
+      </c>
+      <c r="F132" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" t="n">
+        <v>2740233.653965407</v>
+      </c>
+      <c r="E133" t="n">
+        <v>-2740233.653965407</v>
+      </c>
+      <c r="F133" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" t="n">
+        <v>3839645.503585657</v>
+      </c>
+      <c r="E134" t="n">
+        <v>-3839645.503585657</v>
+      </c>
+      <c r="F134" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>0</v>
+      </c>
+      <c r="D135" t="n">
+        <v>4248902.952380952</v>
+      </c>
+      <c r="E135" t="n">
+        <v>-4248902.952380952</v>
+      </c>
+      <c r="F135" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" t="n">
+        <v>24163742.91004469</v>
+      </c>
+      <c r="E136" t="n">
+        <v>-24163742.91004469</v>
+      </c>
+      <c r="F136" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>0</v>
+      </c>
+      <c r="D137" t="n">
+        <v>18899174.40615667</v>
+      </c>
+      <c r="E137" t="n">
+        <v>-18899174.40615667</v>
+      </c>
+      <c r="F137" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" t="n">
+        <v>22449175.76470205</v>
+      </c>
+      <c r="E138" t="n">
+        <v>-22449175.76470205</v>
+      </c>
+      <c r="F138" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Sep-26</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>0</v>
+      </c>
+      <c r="D139" t="n">
+        <v>10658334.49238095</v>
+      </c>
+      <c r="E139" t="n">
+        <v>-10658334.49238095</v>
+      </c>
+      <c r="F139" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>0</v>
+      </c>
+      <c r="D140" t="n">
+        <v>2060918.427395666</v>
+      </c>
+      <c r="E140" t="n">
+        <v>-2060918.427395666</v>
+      </c>
+      <c r="F140" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>0</v>
+      </c>
+      <c r="D141" t="n">
+        <v>3216356.398978495</v>
+      </c>
+      <c r="E141" t="n">
+        <v>-3216356.398978495</v>
+      </c>
+      <c r="F141" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>0</v>
+      </c>
+      <c r="D142" t="n">
+        <v>4552402.952380952</v>
+      </c>
+      <c r="E142" t="n">
+        <v>-4552402.952380952</v>
+      </c>
+      <c r="F142" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>0</v>
+      </c>
+      <c r="D143" t="n">
+        <v>23504509.50771018</v>
+      </c>
+      <c r="E143" t="n">
+        <v>-23504509.50771018</v>
+      </c>
+      <c r="F143" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>0</v>
+      </c>
+      <c r="D144" t="n">
+        <v>20078615.34753704</v>
+      </c>
+      <c r="E144" t="n">
+        <v>-20078615.34753704</v>
+      </c>
+      <c r="F144" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>0</v>
+      </c>
+      <c r="D145" t="n">
+        <v>22648513.31474198</v>
+      </c>
+      <c r="E145" t="n">
+        <v>-22648513.31474198</v>
+      </c>
+      <c r="F145" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Oct-26</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>0</v>
+      </c>
+      <c r="D146" t="n">
+        <v>8288079.832380952</v>
+      </c>
+      <c r="E146" t="n">
+        <v>-8288079.832380952</v>
+      </c>
+      <c r="F146" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0</v>
+      </c>
+      <c r="D147" t="n">
+        <v>3116406.813288246</v>
+      </c>
+      <c r="E147" t="n">
+        <v>-3116406.813288246</v>
+      </c>
+      <c r="F147" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>0</v>
+      </c>
+      <c r="D148" t="n">
+        <v>3247746.489788108</v>
+      </c>
+      <c r="E148" t="n">
+        <v>-3247746.489788108</v>
+      </c>
+      <c r="F148" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>0</v>
+      </c>
+      <c r="D149" t="n">
+        <v>4234534.952380952</v>
+      </c>
+      <c r="E149" t="n">
+        <v>-4234534.952380952</v>
+      </c>
+      <c r="F149" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>0</v>
+      </c>
+      <c r="D150" t="n">
+        <v>23892351.16330291</v>
+      </c>
+      <c r="E150" t="n">
+        <v>-23892351.16330291</v>
+      </c>
+      <c r="F150" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>0</v>
+      </c>
+      <c r="D151" t="n">
+        <v>17771069.28279239</v>
+      </c>
+      <c r="E151" t="n">
+        <v>-17771069.28279239</v>
+      </c>
+      <c r="F151" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>0</v>
+      </c>
+      <c r="D152" t="n">
+        <v>22674603.91006402</v>
+      </c>
+      <c r="E152" t="n">
+        <v>-22674603.91006402</v>
+      </c>
+      <c r="F152" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Nov-26</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>0</v>
+      </c>
+      <c r="D153" t="n">
+        <v>8295856.552380953</v>
+      </c>
+      <c r="E153" t="n">
+        <v>-8295856.552380953</v>
+      </c>
+      <c r="F153" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>0</v>
+      </c>
+      <c r="D154" t="n">
+        <v>4505334.575696514</v>
+      </c>
+      <c r="E154" t="n">
+        <v>-4505334.575696514</v>
+      </c>
+      <c r="F154" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>0</v>
+      </c>
+      <c r="D155" t="n">
+        <v>3409858.838336057</v>
+      </c>
+      <c r="E155" t="n">
+        <v>-3409858.838336057</v>
+      </c>
+      <c r="F155" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>0</v>
+      </c>
+      <c r="D156" t="n">
+        <v>4199902.952380952</v>
+      </c>
+      <c r="E156" t="n">
+        <v>-4199902.952380952</v>
+      </c>
+      <c r="F156" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>0</v>
+      </c>
+      <c r="D157" t="n">
+        <v>24792477.47404118</v>
+      </c>
+      <c r="E157" t="n">
+        <v>-24792477.47404118</v>
+      </c>
+      <c r="F157" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>0</v>
+      </c>
+      <c r="D158" t="n">
+        <v>18760745.56039985</v>
+      </c>
+      <c r="E158" t="n">
+        <v>-18760745.56039985</v>
+      </c>
+      <c r="F158" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>0</v>
+      </c>
+      <c r="D159" t="n">
+        <v>23470015.95171413</v>
+      </c>
+      <c r="E159" t="n">
+        <v>-23470015.95171413</v>
+      </c>
+      <c r="F159" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Dec-26</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>0</v>
+      </c>
+      <c r="D160" t="n">
+        <v>10411892.23238095</v>
+      </c>
+      <c r="E160" t="n">
+        <v>-10411892.23238095</v>
+      </c>
+      <c r="F160" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>0</v>
+      </c>
+      <c r="D161" t="n">
+        <v>3683298.36296571</v>
+      </c>
+      <c r="E161" t="n">
+        <v>-3683298.36296571</v>
+      </c>
+      <c r="F161" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>0</v>
+      </c>
+      <c r="D162" t="n">
+        <v>3456084.406932943</v>
+      </c>
+      <c r="E162" t="n">
+        <v>-3456084.406932943</v>
+      </c>
+      <c r="F162" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>0</v>
+      </c>
+      <c r="D163" t="n">
+        <v>4011730.761904762</v>
+      </c>
+      <c r="E163" t="n">
+        <v>-4011730.761904762</v>
+      </c>
+      <c r="F163" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>0</v>
+      </c>
+      <c r="D164" t="n">
+        <v>23642786.40061948</v>
+      </c>
+      <c r="E164" t="n">
+        <v>-23642786.40061948</v>
+      </c>
+      <c r="F164" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>0</v>
+      </c>
+      <c r="D165" t="n">
+        <v>17390186.84683962</v>
+      </c>
+      <c r="E165" t="n">
+        <v>-17390186.84683962</v>
+      </c>
+      <c r="F165" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>0</v>
+      </c>
+      <c r="D166" t="n">
+        <v>22621936.55925866</v>
+      </c>
+      <c r="E166" t="n">
+        <v>-22621936.55925866</v>
+      </c>
+      <c r="F166" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Jan-27</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>0</v>
+      </c>
+      <c r="D167" t="n">
+        <v>8005196.232380953</v>
+      </c>
+      <c r="E167" t="n">
+        <v>-8005196.232380953</v>
+      </c>
+      <c r="F167" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>0</v>
+      </c>
+      <c r="D168" t="n">
+        <v>3293437.961245519</v>
+      </c>
+      <c r="E168" t="n">
+        <v>-3293437.961245519</v>
+      </c>
+      <c r="F168" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>0</v>
+      </c>
+      <c r="D169" t="n">
+        <v>3477804.401558435</v>
+      </c>
+      <c r="E169" t="n">
+        <v>-3477804.401558435</v>
+      </c>
+      <c r="F169" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>0</v>
+      </c>
+      <c r="D170" t="n">
+        <v>4024230.761904762</v>
+      </c>
+      <c r="E170" t="n">
+        <v>-4024230.761904762</v>
+      </c>
+      <c r="F170" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>0</v>
+      </c>
+      <c r="D171" t="n">
+        <v>24158478.22805225</v>
+      </c>
+      <c r="E171" t="n">
+        <v>-24158478.22805225</v>
+      </c>
+      <c r="F171" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>0</v>
+      </c>
+      <c r="D172" t="n">
+        <v>17379633.51987506</v>
+      </c>
+      <c r="E172" t="n">
+        <v>-17379633.51987506</v>
+      </c>
+      <c r="F172" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>0</v>
+      </c>
+      <c r="D173" t="n">
+        <v>22769135.05253517</v>
+      </c>
+      <c r="E173" t="n">
+        <v>-22769135.05253517</v>
+      </c>
+      <c r="F173" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Feb-27</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>0</v>
+      </c>
+      <c r="D174" t="n">
+        <v>8009468.232380953</v>
+      </c>
+      <c r="E174" t="n">
+        <v>-8009468.232380953</v>
+      </c>
+      <c r="F174" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Advertising &amp; PR</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>0</v>
+      </c>
+      <c r="D175" t="n">
+        <v>1977959.772256132</v>
+      </c>
+      <c r="E175" t="n">
+        <v>-1977959.772256132</v>
+      </c>
+      <c r="F175" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Bad Debt</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>0</v>
+      </c>
+      <c r="D176" t="n">
+        <v>3598284.039392758</v>
+      </c>
+      <c r="E176" t="n">
+        <v>-3598284.039392758</v>
+      </c>
+      <c r="F176" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Consultancy &amp; Other Fees</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>0</v>
+      </c>
+      <c r="D177" t="n">
+        <v>2441557.761904762</v>
+      </c>
+      <c r="E177" t="n">
+        <v>-2441557.761904762</v>
+      </c>
+      <c r="F177" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>0</v>
+      </c>
+      <c r="D178" t="n">
+        <v>27331633.67587252</v>
+      </c>
+      <c r="E178" t="n">
+        <v>-27331633.67587252</v>
+      </c>
+      <c r="F178" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Other Operating Expenses</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>0</v>
+      </c>
+      <c r="D179" t="n">
+        <v>106066711.6235541</v>
+      </c>
+      <c r="E179" t="n">
+        <v>-106066711.6235541</v>
+      </c>
+      <c r="F179" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>0</v>
+      </c>
+      <c r="D180" t="n">
+        <v>74718831.42457715</v>
+      </c>
+      <c r="E180" t="n">
+        <v>-74718831.42457715</v>
+      </c>
+      <c r="F180" t="n">
+        <v>-100</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Mar-27</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Professional</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>0</v>
+      </c>
+      <c r="D181" t="n">
+        <v>9088146.232380953</v>
+      </c>
+      <c r="E181" t="n">
+        <v>-9088146.232380953</v>
+      </c>
+      <c r="F181" t="n">
+        <v>-100</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F144">
-    <filterColumn colId="0" hiddenButton="0" showButton="1">
-      <filters>
-        <filter val="Jul-25"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:F144"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9795,6 +11581,17 @@
   </sheetPr>
   <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.28515625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="5.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="12" bestFit="1" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -12565,6 +14362,12 @@
   </sheetPr>
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="14" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="13.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Rename LY → PY throughout — 'prior year' is TSTT's preferred terminology
- build_board_data.py: Revenue_LY/EBITDA_LY/PAT_LY → _PY; KPI_Summary 'LY' col → 'PY'
- utils/data_loader.py: derived columns _LY → _PY; KPI column renamed; lookup var renamed
- utils/charts.py: kpi_card param vs_ly_pct → vs_py_pct; display label 'LY:' → 'PY:'
- app.py: row['LY'] → row['PY']; vs_ly → vs_py; column refs updated
- pages/1_Financial_Performance.py: column refs and chart titles updated
- pages/3_Cash_CAPEX.py: 'vs LY' → 'vs PY'; DSO/DPO placeholders updated
- pages/8_Financial_Performance_V2.py: EBITDA_Margin_LY → _PY; METRICS and driver blocks updated
- TSTT_Board_Data.xlsx: rebuilt with PY column names

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>LY</t>
+          <t>PY</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3741,17 +3741,17 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Revenue_LY</t>
+          <t>Revenue_PY</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>EBITDA_LY</t>
+          <t>EBITDA_PY</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>PAT_LY</t>
+          <t>PAT_PY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve Consumer V2 donut chart, sparklines, and set jet black background
- Fix donut centre annotation: use domain-derived cx and margin-corrected cy
  so the total label is geometrically centred in the hole
- Add sort=False to pie trace to prevent colour/label mismatches on Postpaid
- Remove Total Revenue Trend bar from V2 right column
- Add inline sparklines to all 5 Row-1 KPI cards in Consumer Sales V2
- Jet black background: config.toml + style.css updated to #000000

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tsttcott-my.sharepoint.com/personal/csimeon_tstt_co_tt/Documents/Financial Analysis/TSTT_Board_Report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_5E7FB0E306739AD202C0CCED51BD4C2C939579DE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88851362-928E-460A-B577-AAF93E3C1EC2}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_5E7FB0E306739AD202C0CCED51BD4C2C939579DE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0C0BBCF-6F5E-4134-A775-CD5BF4D386DC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Summary" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <sheet name="AMPLIA_Commercial" sheetId="12" r:id="rId12"/>
     <sheet name="PnL_Breakdown" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -848,9 +848,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -876,7 +876,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -902,7 +902,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -928,7 +928,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -954,7 +954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -988,9 +988,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:H27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1016,7 +1016,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1062,7 +1062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1131,7 +1131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>26</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1338,7 +1338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1361,7 +1361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1430,7 +1430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -1545,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>8</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>8</v>
       </c>
@@ -1628,9 +1628,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>5052508.66</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>4772772.4800000004</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>4868498.7799999993</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1775,7 +1775,7 @@
         <v>4888500.08</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -1804,7 +1804,7 @@
         <v>4838473.97</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>4184827.09</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -1862,7 +1862,7 @@
         <v>4731653.62</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>4885687.32</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>5015843.0600000015</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -1949,7 +1949,7 @@
         <v>5063916.8599999994</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>10988379.380000001</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -2007,7 +2007,7 @@
         <v>4603785.7300000004</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -2044,9 +2044,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:J12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2110,7 +2110,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2174,7 +2174,7 @@
         <v>1702</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>1732</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>1869</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>1744</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>1615</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -2334,7 +2334,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -2366,7 +2366,7 @@
         <v>1955</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>1738</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -2438,9 +2438,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:AC14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>60277161.446693897</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>60345233.043752059</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2796,7 +2796,7 @@
         <v>57538201.224007033</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>68316247.276720509</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2974,7 +2974,7 @@
         <v>59749496.670891792</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>66232114.599926889</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>66948525.912469313</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>65020418.769918293</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>73151131.008717939</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -3419,7 +3419,7 @@
         <v>70992145.038130015</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>69078251.34582293</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -3597,7 +3597,7 @@
         <v>72567588.15664874</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -3694,9 +3694,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>-3493079.5246898979</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>1614537.304295762</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>2130967.3403671761</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>9013224.3888138775</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -3861,7 +3861,7 @@
         <v>-6211670.3604888832</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -3887,7 +3887,7 @@
         <v>13547997.1464362</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -3913,7 +3913,7 @@
         <v>116276.11797960851</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>1543430.109830589</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -3965,7 +3965,7 @@
         <v>5428866.3605959089</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -3991,7 +3991,7 @@
         <v>837530.04506034299</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -4017,7 +4017,7 @@
         <v>-128382.4449065286</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>9822165.6603516266</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -4086,9 +4086,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -4180,9 +4180,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F145"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4202,7 +4202,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -4222,7 +4222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -4242,7 +4242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -4322,7 +4322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -4362,7 +4362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4402,7 +4402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -4422,7 +4422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -4442,7 +4442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -4482,7 +4482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -4502,7 +4502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -4522,7 +4522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -4562,7 +4562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -4582,7 +4582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -4622,7 +4622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -4662,7 +4662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -4682,7 +4682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -4762,7 +4762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -4822,7 +4822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -4842,7 +4842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -4862,7 +4862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>29</v>
       </c>
@@ -4882,7 +4882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -4902,7 +4902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>29</v>
       </c>
@@ -4922,7 +4922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>30</v>
       </c>
@@ -4942,7 +4942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -4962,7 +4962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>30</v>
       </c>
@@ -4982,7 +4982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -5022,7 +5022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -5042,7 +5042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>31</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>31</v>
       </c>
@@ -5082,7 +5082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>31</v>
       </c>
@@ -5102,7 +5102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>31</v>
       </c>
@@ -5122,7 +5122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>31</v>
       </c>
@@ -5142,7 +5142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>31</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>32</v>
       </c>
@@ -5182,7 +5182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>32</v>
       </c>
@@ -5202,7 +5202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -5222,7 +5222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>32</v>
       </c>
@@ -5242,7 +5242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>32</v>
       </c>
@@ -5262,7 +5262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>32</v>
       </c>
@@ -5282,7 +5282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>33</v>
       </c>
@@ -5302,7 +5302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>33</v>
       </c>
@@ -5322,7 +5322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>33</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>33</v>
       </c>
@@ -5362,7 +5362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>33</v>
       </c>
@@ -5382,7 +5382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>33</v>
       </c>
@@ -5402,7 +5402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>34</v>
       </c>
@@ -5422,7 +5422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>34</v>
       </c>
@@ -5442,7 +5442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>34</v>
       </c>
@@ -5462,7 +5462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>34</v>
       </c>
@@ -5482,7 +5482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>34</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>34</v>
       </c>
@@ -5522,7 +5522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>35</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>35</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>35</v>
       </c>
@@ -5582,7 +5582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>35</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>35</v>
       </c>
@@ -5622,7 +5622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>35</v>
       </c>
@@ -5642,7 +5642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -5662,7 +5662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -5682,7 +5682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -5702,7 +5702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -5722,7 +5722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -5742,7 +5742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -5762,7 +5762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>58</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>58</v>
       </c>
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>58</v>
       </c>
@@ -5813,7 +5813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>58</v>
       </c>
@@ -5830,7 +5830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>58</v>
       </c>
@@ -5847,7 +5847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>58</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>59</v>
       </c>
@@ -5881,7 +5881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>59</v>
       </c>
@@ -5898,7 +5898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>59</v>
       </c>
@@ -5915,7 +5915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>59</v>
       </c>
@@ -5932,7 +5932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>59</v>
       </c>
@@ -5949,7 +5949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>59</v>
       </c>
@@ -5966,7 +5966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>60</v>
       </c>
@@ -5983,7 +5983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>60</v>
       </c>
@@ -6000,7 +6000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>60</v>
       </c>
@@ -6017,7 +6017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>60</v>
       </c>
@@ -6034,7 +6034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>60</v>
       </c>
@@ -6051,7 +6051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>60</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>61</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>61</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>61</v>
       </c>
@@ -6119,7 +6119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>61</v>
       </c>
@@ -6136,7 +6136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>61</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>61</v>
       </c>
@@ -6170,7 +6170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>62</v>
       </c>
@@ -6187,7 +6187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>62</v>
       </c>
@@ -6204,7 +6204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>62</v>
       </c>
@@ -6221,7 +6221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>62</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>62</v>
       </c>
@@ -6255,7 +6255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>62</v>
       </c>
@@ -6272,7 +6272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>63</v>
       </c>
@@ -6289,7 +6289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>63</v>
       </c>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>63</v>
       </c>
@@ -6323,7 +6323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>63</v>
       </c>
@@ -6340,7 +6340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>63</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>63</v>
       </c>
@@ -6374,7 +6374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>64</v>
       </c>
@@ -6391,7 +6391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>64</v>
       </c>
@@ -6408,7 +6408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>64</v>
       </c>
@@ -6425,7 +6425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>64</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>64</v>
       </c>
@@ -6459,7 +6459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>64</v>
       </c>
@@ -6476,7 +6476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>65</v>
       </c>
@@ -6493,7 +6493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>65</v>
       </c>
@@ -6510,7 +6510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>65</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>65</v>
       </c>
@@ -6544,7 +6544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>65</v>
       </c>
@@ -6561,7 +6561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>65</v>
       </c>
@@ -6578,7 +6578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>66</v>
       </c>
@@ -6595,7 +6595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>66</v>
       </c>
@@ -6612,7 +6612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>66</v>
       </c>
@@ -6629,7 +6629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>66</v>
       </c>
@@ -6646,7 +6646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>66</v>
       </c>
@@ -6663,7 +6663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>66</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>67</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>67</v>
       </c>
@@ -6714,7 +6714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>67</v>
       </c>
@@ -6731,7 +6731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>67</v>
       </c>
@@ -6748,7 +6748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>67</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>67</v>
       </c>
@@ -6782,7 +6782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
         <v>68</v>
       </c>
@@ -6799,7 +6799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
         <v>68</v>
       </c>
@@ -6816,7 +6816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>68</v>
       </c>
@@ -6833,7 +6833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>68</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>68</v>
       </c>
@@ -6867,7 +6867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>68</v>
       </c>
@@ -6892,9 +6892,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6917,7 +6917,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -6937,7 +6937,7 @@
         <v>10792000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -6957,7 +6957,7 @@
         <v>23912000</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>14219000</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>24791000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -7017,7 +7017,7 @@
         <v>8949000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -7037,7 +7037,7 @@
         <v>18089000</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -7057,7 +7057,7 @@
         <v>31759000</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -7077,7 +7077,7 @@
         <v>44506000</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -7097,7 +7097,7 @@
         <v>22803000</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -7117,7 +7117,7 @@
         <v>35050000</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>13194000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -7165,9 +7165,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H79"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7193,7 +7203,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -7216,7 +7226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -7239,7 +7249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -7262,7 +7272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -7285,7 +7295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -7308,7 +7318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -7331,7 +7341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -7354,7 +7364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -7377,7 +7387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -7400,7 +7410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -7423,7 +7433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -7446,7 +7456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -7469,7 +7479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -7492,7 +7502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -7515,7 +7525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -7538,7 +7548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -7561,7 +7571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -7584,7 +7594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -7607,7 +7617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -7630,7 +7640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -7653,7 +7663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -7676,7 +7686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -7699,7 +7709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -7722,7 +7732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -7745,7 +7755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -7768,7 +7778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -7791,7 +7801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -7814,7 +7824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -7837,7 +7847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -7860,7 +7870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -7883,7 +7893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -7906,7 +7916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -7929,7 +7939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>29</v>
       </c>
@@ -7952,7 +7962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>29</v>
       </c>
@@ -7975,7 +7985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -7998,7 +8008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>29</v>
       </c>
@@ -8021,7 +8031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>30</v>
       </c>
@@ -8044,7 +8054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -8067,7 +8077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>30</v>
       </c>
@@ -8090,7 +8100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -8113,7 +8123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -8136,7 +8146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -8159,7 +8169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>31</v>
       </c>
@@ -8182,7 +8192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>31</v>
       </c>
@@ -8205,7 +8215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>31</v>
       </c>
@@ -8228,7 +8238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>31</v>
       </c>
@@ -8251,7 +8261,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>31</v>
       </c>
@@ -8274,7 +8284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>31</v>
       </c>
@@ -8297,7 +8307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>32</v>
       </c>
@@ -8320,7 +8330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>32</v>
       </c>
@@ -8343,7 +8353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>32</v>
       </c>
@@ -8366,7 +8376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>32</v>
       </c>
@@ -8389,7 +8399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>32</v>
       </c>
@@ -8412,7 +8422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>32</v>
       </c>
@@ -8435,7 +8445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>33</v>
       </c>
@@ -8458,7 +8468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>33</v>
       </c>
@@ -8481,7 +8491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>33</v>
       </c>
@@ -8504,7 +8514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>33</v>
       </c>
@@ -8527,7 +8537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>33</v>
       </c>
@@ -8550,7 +8560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>33</v>
       </c>
@@ -8573,7 +8583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>34</v>
       </c>
@@ -8596,7 +8606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>34</v>
       </c>
@@ -8619,7 +8629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>34</v>
       </c>
@@ -8642,7 +8652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>34</v>
       </c>
@@ -8665,7 +8675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>34</v>
       </c>
@@ -8688,7 +8698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>34</v>
       </c>
@@ -8711,7 +8721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>35</v>
       </c>
@@ -8734,7 +8744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>35</v>
       </c>
@@ -8757,7 +8767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>35</v>
       </c>
@@ -8780,7 +8790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>35</v>
       </c>
@@ -8803,7 +8813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>35</v>
       </c>
@@ -8826,7 +8836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>35</v>
       </c>
@@ -8849,7 +8859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -8875,7 +8885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -8901,7 +8911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -8927,7 +8937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -8953,7 +8963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -8979,7 +8989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -9013,9 +9023,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:I92"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -9044,7 +9054,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -9070,7 +9080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -9096,7 +9106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -9122,7 +9132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -9148,7 +9158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -9171,7 +9181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -9197,7 +9207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -9223,7 +9233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -9249,7 +9259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -9275,7 +9285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -9301,7 +9311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -9327,7 +9337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -9350,7 +9360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -9376,7 +9386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -9402,7 +9412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -9428,7 +9438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -9454,7 +9464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>26</v>
       </c>
@@ -9480,7 +9490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -9506,7 +9516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -9529,7 +9539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -9555,7 +9565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -9581,7 +9591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -9607,7 +9617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -9633,7 +9643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -9659,7 +9669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -9685,7 +9695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -9708,7 +9718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -9734,7 +9744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -9760,7 +9770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -9786,7 +9796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
@@ -9812,7 +9822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -9838,7 +9848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>28</v>
       </c>
@@ -9864,7 +9874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>28</v>
       </c>
@@ -9887,7 +9897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>28</v>
       </c>
@@ -9913,7 +9923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>28</v>
       </c>
@@ -9939,7 +9949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>29</v>
       </c>
@@ -9965,7 +9975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>29</v>
       </c>
@@ -9991,7 +10001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>29</v>
       </c>
@@ -10017,7 +10027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>29</v>
       </c>
@@ -10043,7 +10053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>29</v>
       </c>
@@ -10066,7 +10076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>29</v>
       </c>
@@ -10092,7 +10102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>29</v>
       </c>
@@ -10118,7 +10128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -10144,7 +10154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -10170,7 +10180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>30</v>
       </c>
@@ -10196,7 +10206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -10222,7 +10232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -10245,7 +10255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -10271,7 +10281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -10297,7 +10307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>31</v>
       </c>
@@ -10323,7 +10333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>31</v>
       </c>
@@ -10349,7 +10359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>31</v>
       </c>
@@ -10375,7 +10385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>31</v>
       </c>
@@ -10401,7 +10411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>31</v>
       </c>
@@ -10424,7 +10434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>31</v>
       </c>
@@ -10450,7 +10460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>31</v>
       </c>
@@ -10476,7 +10486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>32</v>
       </c>
@@ -10502,7 +10512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -10528,7 +10538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>32</v>
       </c>
@@ -10554,7 +10564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>32</v>
       </c>
@@ -10580,7 +10590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>32</v>
       </c>
@@ -10603,7 +10613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>32</v>
       </c>
@@ -10629,7 +10639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>32</v>
       </c>
@@ -10655,7 +10665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>33</v>
       </c>
@@ -10681,7 +10691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>33</v>
       </c>
@@ -10707,7 +10717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>33</v>
       </c>
@@ -10733,7 +10743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>33</v>
       </c>
@@ -10759,7 +10769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>33</v>
       </c>
@@ -10782,7 +10792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>33</v>
       </c>
@@ -10808,7 +10818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>33</v>
       </c>
@@ -10834,7 +10844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>34</v>
       </c>
@@ -10860,7 +10870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>34</v>
       </c>
@@ -10886,7 +10896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>34</v>
       </c>
@@ -10912,7 +10922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>34</v>
       </c>
@@ -10938,7 +10948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>34</v>
       </c>
@@ -10961,7 +10971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>34</v>
       </c>
@@ -10987,7 +10997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>34</v>
       </c>
@@ -11013,7 +11023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>35</v>
       </c>
@@ -11039,7 +11049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>35</v>
       </c>
@@ -11065,7 +11075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>35</v>
       </c>
@@ -11091,7 +11101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>35</v>
       </c>
@@ -11117,7 +11127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>35</v>
       </c>
@@ -11140,7 +11150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>35</v>
       </c>
@@ -11166,7 +11176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>35</v>
       </c>
@@ -11192,7 +11202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -11221,7 +11231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -11250,7 +11260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -11279,7 +11289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -11308,7 +11318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -11334,7 +11344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -11363,7 +11373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>8</v>
       </c>
@@ -11397,9 +11407,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -11427,9 +11437,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>102</v>
       </c>

</xml_diff>

<commit_message>
Postpaid plans donut: add Legacy segment as majority slice
PP_Plans sheet now has 6 rows: Legacy (180K, amber) + 5 active plans (blue shades).
Legacy is the largest segment by design — update Subscribers in that sheet with
actual counts when available.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -18,9 +18,9 @@
     <sheet name="DPDI" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="AMPLIA_Financial" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="AMPLIA_Commercial" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="PnL_Breakdown" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Pre_ARPU_Cats" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="PP_Plans" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="PP_Plans" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="PnL_Breakdown" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Pre_ARPU_Cats" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="WTTx_ARPU_Cats" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
@@ -2342,1337 +2342,102 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CONSUMER SALES_Rev</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>CONSUMER SALES_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>CONSUMER SALES_COS</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>CONSUMER SALES_COS_AOP</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>BUSINESS SALES_Rev</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>BUSINESS SALES_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>BUSINESS SALES_COS</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>BUSINESS SALES_COS_AOP</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>AMPLIA_Rev</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>AMPLIA_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>AMPLIA_COS</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>AMPLIA_COS_AOP</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>DPDI_Rev</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>DPDI_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>DPDI_COS</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>DPDI_COS_AOP</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>OTHER_Rev</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>OTHER_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>OTHER_COS</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>OTHER_COS_AOP</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Rev</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Total_Rev_AOP</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Total_COS</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Total_COS_AOP</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Total_OPEX</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>Total_OPEX_AOP</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>EBITDA_AOP</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Subscribers</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Monthly_Fee_TTD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Legacy</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>91096868.77000003</v>
+        <v>180000</v>
       </c>
       <c r="C2" t="n">
-        <v>91861724.33722802</v>
-      </c>
-      <c r="D2" t="n">
-        <v>14010859.5</v>
-      </c>
-      <c r="E2" t="n">
-        <v>14694559</v>
-      </c>
-      <c r="F2" t="n">
-        <v>46030788.94</v>
-      </c>
-      <c r="G2" t="n">
-        <v>46038101.31160618</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2993618.490000005</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3914465.000221079</v>
-      </c>
-      <c r="J2" t="n">
-        <v>25447329.81</v>
-      </c>
-      <c r="K2" t="n">
-        <v>25306707</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5052508.66</v>
-      </c>
-      <c r="M2" t="n">
-        <v>5424966.671355191</v>
-      </c>
-      <c r="N2" t="n">
-        <v>938594.01</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>217680.38</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>-2000000</v>
-      </c>
-      <c r="S2" t="n">
-        <v>-2699339.957355191</v>
-      </c>
-      <c r="T2" t="n">
-        <v>-1834298</v>
-      </c>
-      <c r="U2" t="n">
-        <v>-2173327.611799635</v>
-      </c>
-      <c r="V2" t="n">
-        <v>161513581.53</v>
-      </c>
-      <c r="W2" t="n">
-        <v>161455631.371479</v>
-      </c>
-      <c r="X2" t="n">
-        <v>20440369.03</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>22095623.50577664</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>70534458.91</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>79142846.41900846</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>70625668.58000004</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>60277161.4466939</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>May-25</t>
+          <t>Basic Voice</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>90216607.98999998</v>
+        <v>45000</v>
       </c>
       <c r="C3" t="n">
-        <v>94477769.34541556</v>
-      </c>
-      <c r="D3" t="n">
-        <v>14495304.21</v>
-      </c>
-      <c r="E3" t="n">
-        <v>17949064</v>
-      </c>
-      <c r="F3" t="n">
-        <v>49130568.39000001</v>
-      </c>
-      <c r="G3" t="n">
-        <v>46867653.30865601</v>
-      </c>
-      <c r="H3" t="n">
-        <v>3677532.320000003</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3957438.122569739</v>
-      </c>
-      <c r="J3" t="n">
-        <v>26113220.11</v>
-      </c>
-      <c r="K3" t="n">
-        <v>25695738</v>
-      </c>
-      <c r="L3" t="n">
-        <v>4772772.48</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5536017.290862304</v>
-      </c>
-      <c r="N3" t="n">
-        <v>1487994.94</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>567680.38</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>-2760275.319999993</v>
-      </c>
-      <c r="S3" t="n">
-        <v>-1925581.206862304</v>
-      </c>
-      <c r="T3" t="n">
-        <v>-2007753</v>
-      </c>
-      <c r="U3" t="n">
-        <v>-2193497.231306748</v>
-      </c>
-      <c r="V3" t="n">
-        <v>164188116.11</v>
-      </c>
-      <c r="W3" t="n">
-        <v>166064018.1272093</v>
-      </c>
-      <c r="X3" t="n">
-        <v>21505536.39</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>25483982.6281253</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>75810568.88496403</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>80294802.45533194</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>66878419.69503598</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>60345233.04375206</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jun-25</t>
+          <t>Basic Data</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>92076140.39</v>
+        <v>38000</v>
       </c>
       <c r="C4" t="n">
-        <v>95355430.26794931</v>
-      </c>
-      <c r="D4" t="n">
-        <v>14320378.37</v>
-      </c>
-      <c r="E4" t="n">
-        <v>17149115</v>
-      </c>
-      <c r="F4" t="n">
-        <v>47973222.28</v>
-      </c>
-      <c r="G4" t="n">
-        <v>49271362.95392575</v>
-      </c>
-      <c r="H4" t="n">
-        <v>4074876.499999999</v>
-      </c>
-      <c r="I4" t="n">
-        <v>5669547.26212224</v>
-      </c>
-      <c r="J4" t="n">
-        <v>26264263.11999999</v>
-      </c>
-      <c r="K4" t="n">
-        <v>26117859</v>
-      </c>
-      <c r="L4" t="n">
-        <v>4868498.779999999</v>
-      </c>
-      <c r="M4" t="n">
-        <v>5667066.271218739</v>
-      </c>
-      <c r="N4" t="n">
-        <v>849467.6</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>217680.38</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>-2099197.270000011</v>
-      </c>
-      <c r="S4" t="n">
-        <v>-1873232.94721874</v>
-      </c>
-      <c r="T4" t="n">
-        <v>-2506000</v>
-      </c>
-      <c r="U4" t="n">
-        <v>-2213383.211663184</v>
-      </c>
-      <c r="V4" t="n">
-        <v>165063896.12</v>
-      </c>
-      <c r="W4" t="n">
-        <v>169808297.9546563</v>
-      </c>
-      <c r="X4" t="n">
-        <v>20975434.03</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>26499213.7676778</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>61139026.484</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>85830882.96297152</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>82957229.07600001</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>57538201.22400703</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jul-25</t>
+          <t>Standard Bundle</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>92352581.47000001</v>
+        <v>22000</v>
       </c>
       <c r="C5" t="n">
-        <v>93050892.72757138</v>
-      </c>
-      <c r="D5" t="n">
-        <v>12750826.02</v>
-      </c>
-      <c r="E5" t="n">
-        <v>14026249</v>
-      </c>
-      <c r="F5" t="n">
-        <v>47587833.92</v>
-      </c>
-      <c r="G5" t="n">
-        <v>57191021.8726786</v>
-      </c>
-      <c r="H5" t="n">
-        <v>4168335.999999999</v>
-      </c>
-      <c r="I5" t="n">
-        <v>9034393.60408327</v>
-      </c>
-      <c r="J5" t="n">
-        <v>26813033.17</v>
-      </c>
-      <c r="K5" t="n">
-        <v>26548290</v>
-      </c>
-      <c r="L5" t="n">
-        <v>4888500.08</v>
-      </c>
-      <c r="M5" t="n">
-        <v>5903059.725788871</v>
-      </c>
-      <c r="N5" t="n">
-        <v>811866.53</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>194375</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>-2103522.920000017</v>
-      </c>
-      <c r="S5" t="n">
-        <v>-1884423.78178887</v>
-      </c>
-      <c r="T5" t="n">
-        <v>-1959028</v>
-      </c>
-      <c r="U5" t="n">
-        <v>-2231587.666233315</v>
-      </c>
-      <c r="V5" t="n">
-        <v>165461792.17</v>
-      </c>
-      <c r="W5" t="n">
-        <v>175868411.7184611</v>
-      </c>
-      <c r="X5" t="n">
-        <v>20043009.1</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>26946489.66363882</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>69348866.35740462</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>80665674.77810179</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>77217920.58259538</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>68316247.27672051</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Aug-25</t>
+          <t>Premium Bundle</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>91710972.35000001</v>
+        <v>15000</v>
       </c>
       <c r="C6" t="n">
-        <v>94922246.92634216</v>
-      </c>
-      <c r="D6" t="n">
-        <v>14354491.13</v>
-      </c>
-      <c r="E6" t="n">
-        <v>14258018</v>
-      </c>
-      <c r="F6" t="n">
-        <v>50292629.49</v>
-      </c>
-      <c r="G6" t="n">
-        <v>48659101.64179683</v>
-      </c>
-      <c r="H6" t="n">
-        <v>6465935.41</v>
-      </c>
-      <c r="I6" t="n">
-        <v>12013341.36505904</v>
-      </c>
-      <c r="J6" t="n">
-        <v>26736564.21</v>
-      </c>
-      <c r="K6" t="n">
-        <v>27145842</v>
-      </c>
-      <c r="L6" t="n">
-        <v>4838473.97</v>
-      </c>
-      <c r="M6" t="n">
-        <v>6177159.525720645</v>
-      </c>
-      <c r="N6" t="n">
-        <v>1175208.19</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>194375</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>-1801235.030000001</v>
-      </c>
-      <c r="S6" t="n">
-        <v>-1913793.101720645</v>
-      </c>
-      <c r="T6" t="n">
-        <v>-1992385</v>
-      </c>
-      <c r="U6" t="n">
-        <v>-2252756.46616509</v>
-      </c>
-      <c r="V6" t="n">
-        <v>168114139.21</v>
-      </c>
-      <c r="W6" t="n">
-        <v>169776028.3664184</v>
-      </c>
-      <c r="X6" t="n">
-        <v>23860890.50999999</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>30410137.4246146</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>57139294.3366566</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>79676394.27091196</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>87175279.61334342</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>59749496.67089179</v>
+        <v>399</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sep-25</t>
+          <t>Enterprise</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>90128359.70000002</v>
+        <v>8000</v>
       </c>
       <c r="C7" t="n">
-        <v>95256419.87762924</v>
-      </c>
-      <c r="D7" t="n">
-        <v>12401311.8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>14335147</v>
-      </c>
-      <c r="F7" t="n">
-        <v>49694116.7</v>
-      </c>
-      <c r="G7" t="n">
-        <v>55726352.92198627</v>
-      </c>
-      <c r="H7" t="n">
-        <v>3994895.449999998</v>
-      </c>
-      <c r="I7" t="n">
-        <v>10118915.56281924</v>
-      </c>
-      <c r="J7" t="n">
-        <v>26178595.18</v>
-      </c>
-      <c r="K7" t="n">
-        <v>27695774</v>
-      </c>
-      <c r="L7" t="n">
-        <v>4184827.09</v>
-      </c>
-      <c r="M7" t="n">
-        <v>6376459.743183928</v>
-      </c>
-      <c r="N7" t="n">
-        <v>931282.51</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>194375</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>-1929293.910000026</v>
-      </c>
-      <c r="S7" t="n">
-        <v>-1922257.799183928</v>
-      </c>
-      <c r="T7" t="n">
-        <v>3383837.23</v>
-      </c>
-      <c r="U7" t="n">
-        <v>-2269421.683628372</v>
-      </c>
-      <c r="V7" t="n">
-        <v>165003060.18</v>
-      </c>
-      <c r="W7" t="n">
-        <v>177718919.9004316</v>
-      </c>
-      <c r="X7" t="n">
-        <v>24159246.57</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>28775475.6223748</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>88389572.78</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>82771329.67812991</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>53343312.77000001</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>66232114.59992689</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Oct-25</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>90463809.88</v>
-      </c>
-      <c r="C8" t="n">
-        <v>98674774.79495525</v>
-      </c>
-      <c r="D8" t="n">
-        <v>12708159.02</v>
-      </c>
-      <c r="E8" t="n">
-        <v>21300316</v>
-      </c>
-      <c r="F8" t="n">
-        <v>47588262.2</v>
-      </c>
-      <c r="G8" t="n">
-        <v>50227856.88656416</v>
-      </c>
-      <c r="H8" t="n">
-        <v>3634572.31</v>
-      </c>
-      <c r="I8" t="n">
-        <v>4313561.95097963</v>
-      </c>
-      <c r="J8" t="n">
-        <v>27643427.7</v>
-      </c>
-      <c r="K8" t="n">
-        <v>28012879</v>
-      </c>
-      <c r="L8" t="n">
-        <v>4731653.62</v>
-      </c>
-      <c r="M8" t="n">
-        <v>6614449.37043488</v>
-      </c>
-      <c r="N8" t="n">
-        <v>1079682.51</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>194375</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>-2547000</v>
-      </c>
-      <c r="S8" t="n">
-        <v>-1940573.426434881</v>
-      </c>
-      <c r="T8" t="n">
-        <v>-2298255</v>
-      </c>
-      <c r="U8" t="n">
-        <v>-2287737.310879325</v>
-      </c>
-      <c r="V8" t="n">
-        <v>164228182.29</v>
-      </c>
-      <c r="W8" t="n">
-        <v>176668068.1550846</v>
-      </c>
-      <c r="X8" t="n">
-        <v>18970504.95</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>30382465.01053519</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>57673660.21000001</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>79397077.23208006</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>87917309.37999997</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>66948525.91246931</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Nov-25</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>88902786.52</v>
-      </c>
-      <c r="C9" t="n">
-        <v>101914509.4918081</v>
-      </c>
-      <c r="D9" t="n">
-        <v>14703578.64</v>
-      </c>
-      <c r="E9" t="n">
-        <v>20616008</v>
-      </c>
-      <c r="F9" t="n">
-        <v>46360935.73</v>
-      </c>
-      <c r="G9" t="n">
-        <v>62508806.64368133</v>
-      </c>
-      <c r="H9" t="n">
-        <v>3859427.17</v>
-      </c>
-      <c r="I9" t="n">
-        <v>15348644.75734568</v>
-      </c>
-      <c r="J9" t="n">
-        <v>27356236.08</v>
-      </c>
-      <c r="K9" t="n">
-        <v>28597259</v>
-      </c>
-      <c r="L9" t="n">
-        <v>4885687.32</v>
-      </c>
-      <c r="M9" t="n">
-        <v>6872938.37913241</v>
-      </c>
-      <c r="N9" t="n">
-        <v>2157709.42</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>1265375</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>-2639467.669999987</v>
-      </c>
-      <c r="S9" t="n">
-        <v>-1960946.43513241</v>
-      </c>
-      <c r="T9" t="n">
-        <v>-2476148</v>
-      </c>
-      <c r="U9" t="n">
-        <v>-2308110.319576854</v>
-      </c>
-      <c r="V9" t="n">
-        <v>162138200.08</v>
-      </c>
-      <c r="W9" t="n">
-        <v>192827759.600357</v>
-      </c>
-      <c r="X9" t="n">
-        <v>22237920.13</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>40971355.81690125</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>83238334.97</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>86895985.01353751</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>55622267.49000001</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>65020418.76991829</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Dec-25</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>92056924.37999998</v>
-      </c>
-      <c r="C10" t="n">
-        <v>105112539.7619839</v>
-      </c>
-      <c r="D10" t="n">
-        <v>13669721.21</v>
-      </c>
-      <c r="E10" t="n">
-        <v>24118315</v>
-      </c>
-      <c r="F10" t="n">
-        <v>53126006.13</v>
-      </c>
-      <c r="G10" t="n">
-        <v>64564850.52355281</v>
-      </c>
-      <c r="H10" t="n">
-        <v>9149765.82</v>
-      </c>
-      <c r="I10" t="n">
-        <v>8733145.425684026</v>
-      </c>
-      <c r="J10" t="n">
-        <v>26941579.35</v>
-      </c>
-      <c r="K10" t="n">
-        <v>28975873</v>
-      </c>
-      <c r="L10" t="n">
-        <v>5015843.060000001</v>
-      </c>
-      <c r="M10" t="n">
-        <v>7145591.801489527</v>
-      </c>
-      <c r="N10" t="n">
-        <v>53778662.25</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>45087125</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>-2037195.75999999</v>
-      </c>
-      <c r="S10" t="n">
-        <v>-1983866.857489527</v>
-      </c>
-      <c r="T10" t="n">
-        <v>-2653712</v>
-      </c>
-      <c r="U10" t="n">
-        <v>-2331030.741933972</v>
-      </c>
-      <c r="V10" t="n">
-        <v>223865976.35</v>
-      </c>
-      <c r="W10" t="n">
-        <v>198731718.3280472</v>
-      </c>
-      <c r="X10" t="n">
-        <v>70268743.09</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>38137896.48523958</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>85821328.38999999</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>87502690.83408965</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>67899678.31999999</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>73151131.00871794</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Jan-26</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>89570651.43000001</v>
-      </c>
-      <c r="C11" t="n">
-        <v>94892293.2192031</v>
-      </c>
-      <c r="D11" t="n">
-        <v>12704569.97</v>
-      </c>
-      <c r="E11" t="n">
-        <v>14100869.41</v>
-      </c>
-      <c r="F11" t="n">
-        <v>45833455.48</v>
-      </c>
-      <c r="G11" t="n">
-        <v>55775449.37978129</v>
-      </c>
-      <c r="H11" t="n">
-        <v>5159112.889999998</v>
-      </c>
-      <c r="I11" t="n">
-        <v>8740611.206033947</v>
-      </c>
-      <c r="J11" t="n">
-        <v>26995058.56189249</v>
-      </c>
-      <c r="K11" t="n">
-        <v>29393218</v>
-      </c>
-      <c r="L11" t="n">
-        <v>5063916.859999999</v>
-      </c>
-      <c r="M11" t="n">
-        <v>7317661.119463768</v>
-      </c>
-      <c r="N11" t="n">
-        <v>29378388.9</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>24393875</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>-2351353.810000002</v>
-      </c>
-      <c r="S11" t="n">
-        <v>-1996431.175463768</v>
-      </c>
-      <c r="T11" t="n">
-        <v>-2773000</v>
-      </c>
-      <c r="U11" t="n">
-        <v>-2343595.059908213</v>
-      </c>
-      <c r="V11" t="n">
-        <v>189426200.5618925</v>
-      </c>
-      <c r="W11" t="n">
-        <v>181170857.5901873</v>
-      </c>
-      <c r="X11" t="n">
-        <v>44548474.72</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>28955637.27558951</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>65462556.84424999</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>81283075.27646777</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>79538114.5476425</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>70992145.03813002</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Feb-26</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>86627198.53</v>
-      </c>
-      <c r="C12" t="n">
-        <v>96008362.93721315</v>
-      </c>
-      <c r="D12" t="n">
-        <v>12420253.18</v>
-      </c>
-      <c r="E12" t="n">
-        <v>18468843.41</v>
-      </c>
-      <c r="F12" t="n">
-        <v>49594614.91</v>
-      </c>
-      <c r="G12" t="n">
-        <v>52209344.05719531</v>
-      </c>
-      <c r="H12" t="n">
-        <v>4697652.45</v>
-      </c>
-      <c r="I12" t="n">
-        <v>3764030.682719573</v>
-      </c>
-      <c r="J12" t="n">
-        <v>27244862.09</v>
-      </c>
-      <c r="K12" t="n">
-        <v>29880629</v>
-      </c>
-      <c r="L12" t="n">
-        <v>10988379.38</v>
-      </c>
-      <c r="M12" t="n">
-        <v>7495389.334991091</v>
-      </c>
-      <c r="N12" t="n">
-        <v>53371865.19</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
-        <v>44301206.73</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>-810386.6299999952</v>
-      </c>
-      <c r="S12" t="n">
-        <v>-2004757.390991091</v>
-      </c>
-      <c r="T12" t="n">
-        <v>-905000</v>
-      </c>
-      <c r="U12" t="n">
-        <v>-2351921.275435536</v>
-      </c>
-      <c r="V12" t="n">
-        <v>216028154.09</v>
-      </c>
-      <c r="W12" t="n">
-        <v>179252406.770084</v>
-      </c>
-      <c r="X12" t="n">
-        <v>71502491.73999999</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>28516432.75227513</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>66132145.10608834</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>81717722.67198595</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>78514328.51391169</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>69078251.34582293</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mar-26</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>108214511.69</v>
-      </c>
-      <c r="C13" t="n">
-        <v>94631079.54768565</v>
-      </c>
-      <c r="D13" t="n">
-        <v>13045142.61</v>
-      </c>
-      <c r="E13" t="n">
-        <v>17868311</v>
-      </c>
-      <c r="F13" t="n">
-        <v>82925659.89</v>
-      </c>
-      <c r="G13" t="n">
-        <v>66884533.84582798</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1836751.030000004</v>
-      </c>
-      <c r="I13" t="n">
-        <v>14313238.62119834</v>
-      </c>
-      <c r="J13" t="n">
-        <v>29642976.66</v>
-      </c>
-      <c r="K13" t="n">
-        <v>30155964</v>
-      </c>
-      <c r="L13" t="n">
-        <v>4603785.73</v>
-      </c>
-      <c r="M13" t="n">
-        <v>7734181.205156771</v>
-      </c>
-      <c r="N13" t="n">
-        <v>908753.9300000001</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>243119.99</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>-2103099.51000002</v>
-      </c>
-      <c r="S13" t="n">
-        <v>-2985901.491156771</v>
-      </c>
-      <c r="T13" t="n">
-        <v>-14457484.17</v>
-      </c>
-      <c r="U13" t="n">
-        <v>-2365427.145601215</v>
-      </c>
-      <c r="V13" t="n">
-        <v>219588802.66</v>
-      </c>
-      <c r="W13" t="n">
-        <v>199291615.1690235</v>
-      </c>
-      <c r="X13" t="n">
-        <v>5271315.190000005</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>40490394.2807539</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>111963280.11</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>86293632.73162086</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>107853458.94</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>72567588.15664874</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Apr-26</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>91096868.77000003</v>
-      </c>
-      <c r="C14" t="n">
-        <v>80274532.4636035</v>
-      </c>
-      <c r="D14" t="n">
-        <v>14010859.5</v>
-      </c>
-      <c r="E14" t="n">
-        <v>10442347.08371727</v>
-      </c>
-      <c r="F14" t="n">
-        <v>46030788.94</v>
-      </c>
-      <c r="G14" t="n">
-        <v>46530148.5645342</v>
-      </c>
-      <c r="H14" t="n">
-        <v>2993618.490000005</v>
-      </c>
-      <c r="I14" t="n">
-        <v>3881417.21134247</v>
-      </c>
-      <c r="J14" t="n">
-        <v>25447329.81</v>
-      </c>
-      <c r="K14" t="n">
-        <v>28894159.2091278</v>
-      </c>
-      <c r="L14" t="n">
-        <v>5052508.66</v>
-      </c>
-      <c r="M14" t="n">
-        <v>5142998.307669034</v>
-      </c>
-      <c r="N14" t="n">
-        <v>938594.01</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>217680.38</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>-2000000</v>
-      </c>
-      <c r="S14" t="n">
-        <v>-2953301.1165</v>
-      </c>
-      <c r="T14" t="n">
-        <v>-1834298</v>
-      </c>
-      <c r="U14" t="n">
-        <v>-2217682.8665</v>
-      </c>
-      <c r="V14" t="n">
-        <v>161513581.53</v>
-      </c>
-      <c r="W14" t="n">
-        <v>153681628.0207655</v>
-      </c>
-      <c r="X14" t="n">
-        <v>20440369.03</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>17464854.98622877</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>70534458.91</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>78962885.94843617</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>70625668.58000004</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>57308900.91610059</v>
+        <v>699</v>
       </c>
     </row>
   </sheetData>
@@ -3686,99 +2451,1337 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:AC14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Subscribers</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>ARPU_Band_TTD</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_Rev</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_COS</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>CONSUMER SALES_COS_AOP</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_Rev</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_COS</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BUSINESS SALES_COS_AOP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_Rev</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_COS</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>AMPLIA_COS_AOP</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_Rev</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_COS</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>DPDI_COS_AOP</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_Rev</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_COS</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_COS_AOP</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Rev</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Total_Rev_AOP</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Total_COS</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Total_COS_AOP</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Total_OPEX</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Total_OPEX_AOP</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>EBITDA_AOP</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Very Low</t>
+          <t>Apr-25</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>220000</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>&lt; $50</t>
-        </is>
+        <v>91096868.77000003</v>
+      </c>
+      <c r="C2" t="n">
+        <v>91861724.33722802</v>
+      </c>
+      <c r="D2" t="n">
+        <v>14010859.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14694559</v>
+      </c>
+      <c r="F2" t="n">
+        <v>46030788.94</v>
+      </c>
+      <c r="G2" t="n">
+        <v>46038101.31160618</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2993618.490000005</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3914465.000221079</v>
+      </c>
+      <c r="J2" t="n">
+        <v>25447329.81</v>
+      </c>
+      <c r="K2" t="n">
+        <v>25306707</v>
+      </c>
+      <c r="L2" t="n">
+        <v>5052508.66</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5424966.671355191</v>
+      </c>
+      <c r="N2" t="n">
+        <v>938594.01</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="S2" t="n">
+        <v>-2699339.957355191</v>
+      </c>
+      <c r="T2" t="n">
+        <v>-1834298</v>
+      </c>
+      <c r="U2" t="n">
+        <v>-2173327.611799635</v>
+      </c>
+      <c r="V2" t="n">
+        <v>161513581.53</v>
+      </c>
+      <c r="W2" t="n">
+        <v>161455631.371479</v>
+      </c>
+      <c r="X2" t="n">
+        <v>20440369.03</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>22095623.50577664</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>70534458.91</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>79142846.41900846</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>70625668.58000004</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>60277161.4466939</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>May-25</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>185000</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>$50 - $100</t>
-        </is>
+        <v>90216607.98999998</v>
+      </c>
+      <c r="C3" t="n">
+        <v>94477769.34541556</v>
+      </c>
+      <c r="D3" t="n">
+        <v>14495304.21</v>
+      </c>
+      <c r="E3" t="n">
+        <v>17949064</v>
+      </c>
+      <c r="F3" t="n">
+        <v>49130568.39000001</v>
+      </c>
+      <c r="G3" t="n">
+        <v>46867653.30865601</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3677532.320000003</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3957438.122569739</v>
+      </c>
+      <c r="J3" t="n">
+        <v>26113220.11</v>
+      </c>
+      <c r="K3" t="n">
+        <v>25695738</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4772772.48</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5536017.290862304</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1487994.94</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>567680.38</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>-2760275.319999993</v>
+      </c>
+      <c r="S3" t="n">
+        <v>-1925581.206862304</v>
+      </c>
+      <c r="T3" t="n">
+        <v>-2007753</v>
+      </c>
+      <c r="U3" t="n">
+        <v>-2193497.231306748</v>
+      </c>
+      <c r="V3" t="n">
+        <v>164188116.11</v>
+      </c>
+      <c r="W3" t="n">
+        <v>166064018.1272093</v>
+      </c>
+      <c r="X3" t="n">
+        <v>21505536.39</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>25483982.6281253</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>75810568.88496403</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>80294802.45533194</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>66878419.69503598</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>60345233.04375206</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Jun-25</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>130000</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>$101 - $200</t>
-        </is>
+        <v>92076140.39</v>
+      </c>
+      <c r="C4" t="n">
+        <v>95355430.26794931</v>
+      </c>
+      <c r="D4" t="n">
+        <v>14320378.37</v>
+      </c>
+      <c r="E4" t="n">
+        <v>17149115</v>
+      </c>
+      <c r="F4" t="n">
+        <v>47973222.28</v>
+      </c>
+      <c r="G4" t="n">
+        <v>49271362.95392575</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4074876.499999999</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5669547.26212224</v>
+      </c>
+      <c r="J4" t="n">
+        <v>26264263.11999999</v>
+      </c>
+      <c r="K4" t="n">
+        <v>26117859</v>
+      </c>
+      <c r="L4" t="n">
+        <v>4868498.779999999</v>
+      </c>
+      <c r="M4" t="n">
+        <v>5667066.271218739</v>
+      </c>
+      <c r="N4" t="n">
+        <v>849467.6</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>-2099197.270000011</v>
+      </c>
+      <c r="S4" t="n">
+        <v>-1873232.94721874</v>
+      </c>
+      <c r="T4" t="n">
+        <v>-2506000</v>
+      </c>
+      <c r="U4" t="n">
+        <v>-2213383.211663184</v>
+      </c>
+      <c r="V4" t="n">
+        <v>165063896.12</v>
+      </c>
+      <c r="W4" t="n">
+        <v>169808297.9546563</v>
+      </c>
+      <c r="X4" t="n">
+        <v>20975434.03</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>26499213.7676778</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>61139026.484</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>85830882.96297152</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>82957229.07600001</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>57538201.22400703</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Jul-25</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60000</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>$201 - $400</t>
-        </is>
+        <v>92352581.47000001</v>
+      </c>
+      <c r="C5" t="n">
+        <v>93050892.72757138</v>
+      </c>
+      <c r="D5" t="n">
+        <v>12750826.02</v>
+      </c>
+      <c r="E5" t="n">
+        <v>14026249</v>
+      </c>
+      <c r="F5" t="n">
+        <v>47587833.92</v>
+      </c>
+      <c r="G5" t="n">
+        <v>57191021.8726786</v>
+      </c>
+      <c r="H5" t="n">
+        <v>4168335.999999999</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9034393.60408327</v>
+      </c>
+      <c r="J5" t="n">
+        <v>26813033.17</v>
+      </c>
+      <c r="K5" t="n">
+        <v>26548290</v>
+      </c>
+      <c r="L5" t="n">
+        <v>4888500.08</v>
+      </c>
+      <c r="M5" t="n">
+        <v>5903059.725788871</v>
+      </c>
+      <c r="N5" t="n">
+        <v>811866.53</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>-2103522.920000017</v>
+      </c>
+      <c r="S5" t="n">
+        <v>-1884423.78178887</v>
+      </c>
+      <c r="T5" t="n">
+        <v>-1959028</v>
+      </c>
+      <c r="U5" t="n">
+        <v>-2231587.666233315</v>
+      </c>
+      <c r="V5" t="n">
+        <v>165461792.17</v>
+      </c>
+      <c r="W5" t="n">
+        <v>175868411.7184611</v>
+      </c>
+      <c r="X5" t="n">
+        <v>20043009.1</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>26946489.66363882</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>69348866.35740462</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>80665674.77810179</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>77217920.58259538</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>68316247.27672051</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Very High</t>
+          <t>Aug-25</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25000</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>&gt; $400</t>
-        </is>
+        <v>91710972.35000001</v>
+      </c>
+      <c r="C6" t="n">
+        <v>94922246.92634216</v>
+      </c>
+      <c r="D6" t="n">
+        <v>14354491.13</v>
+      </c>
+      <c r="E6" t="n">
+        <v>14258018</v>
+      </c>
+      <c r="F6" t="n">
+        <v>50292629.49</v>
+      </c>
+      <c r="G6" t="n">
+        <v>48659101.64179683</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6465935.41</v>
+      </c>
+      <c r="I6" t="n">
+        <v>12013341.36505904</v>
+      </c>
+      <c r="J6" t="n">
+        <v>26736564.21</v>
+      </c>
+      <c r="K6" t="n">
+        <v>27145842</v>
+      </c>
+      <c r="L6" t="n">
+        <v>4838473.97</v>
+      </c>
+      <c r="M6" t="n">
+        <v>6177159.525720645</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1175208.19</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>-1801235.030000001</v>
+      </c>
+      <c r="S6" t="n">
+        <v>-1913793.101720645</v>
+      </c>
+      <c r="T6" t="n">
+        <v>-1992385</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-2252756.46616509</v>
+      </c>
+      <c r="V6" t="n">
+        <v>168114139.21</v>
+      </c>
+      <c r="W6" t="n">
+        <v>169776028.3664184</v>
+      </c>
+      <c r="X6" t="n">
+        <v>23860890.50999999</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>30410137.4246146</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>57139294.3366566</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>79676394.27091196</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>87175279.61334342</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>59749496.67089179</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sep-25</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>90128359.70000002</v>
+      </c>
+      <c r="C7" t="n">
+        <v>95256419.87762924</v>
+      </c>
+      <c r="D7" t="n">
+        <v>12401311.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>14335147</v>
+      </c>
+      <c r="F7" t="n">
+        <v>49694116.7</v>
+      </c>
+      <c r="G7" t="n">
+        <v>55726352.92198627</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3994895.449999998</v>
+      </c>
+      <c r="I7" t="n">
+        <v>10118915.56281924</v>
+      </c>
+      <c r="J7" t="n">
+        <v>26178595.18</v>
+      </c>
+      <c r="K7" t="n">
+        <v>27695774</v>
+      </c>
+      <c r="L7" t="n">
+        <v>4184827.09</v>
+      </c>
+      <c r="M7" t="n">
+        <v>6376459.743183928</v>
+      </c>
+      <c r="N7" t="n">
+        <v>931282.51</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-1929293.910000026</v>
+      </c>
+      <c r="S7" t="n">
+        <v>-1922257.799183928</v>
+      </c>
+      <c r="T7" t="n">
+        <v>3383837.23</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-2269421.683628372</v>
+      </c>
+      <c r="V7" t="n">
+        <v>165003060.18</v>
+      </c>
+      <c r="W7" t="n">
+        <v>177718919.9004316</v>
+      </c>
+      <c r="X7" t="n">
+        <v>24159246.57</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>28775475.6223748</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>88389572.78</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>82771329.67812991</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>53343312.77000001</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>66232114.59992689</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Oct-25</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>90463809.88</v>
+      </c>
+      <c r="C8" t="n">
+        <v>98674774.79495525</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12708159.02</v>
+      </c>
+      <c r="E8" t="n">
+        <v>21300316</v>
+      </c>
+      <c r="F8" t="n">
+        <v>47588262.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>50227856.88656416</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3634572.31</v>
+      </c>
+      <c r="I8" t="n">
+        <v>4313561.95097963</v>
+      </c>
+      <c r="J8" t="n">
+        <v>27643427.7</v>
+      </c>
+      <c r="K8" t="n">
+        <v>28012879</v>
+      </c>
+      <c r="L8" t="n">
+        <v>4731653.62</v>
+      </c>
+      <c r="M8" t="n">
+        <v>6614449.37043488</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1079682.51</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>194375</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>-2547000</v>
+      </c>
+      <c r="S8" t="n">
+        <v>-1940573.426434881</v>
+      </c>
+      <c r="T8" t="n">
+        <v>-2298255</v>
+      </c>
+      <c r="U8" t="n">
+        <v>-2287737.310879325</v>
+      </c>
+      <c r="V8" t="n">
+        <v>164228182.29</v>
+      </c>
+      <c r="W8" t="n">
+        <v>176668068.1550846</v>
+      </c>
+      <c r="X8" t="n">
+        <v>18970504.95</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>30382465.01053519</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>57673660.21000001</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>79397077.23208006</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>87917309.37999997</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>66948525.91246931</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>88902786.52</v>
+      </c>
+      <c r="C9" t="n">
+        <v>101914509.4918081</v>
+      </c>
+      <c r="D9" t="n">
+        <v>14703578.64</v>
+      </c>
+      <c r="E9" t="n">
+        <v>20616008</v>
+      </c>
+      <c r="F9" t="n">
+        <v>46360935.73</v>
+      </c>
+      <c r="G9" t="n">
+        <v>62508806.64368133</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3859427.17</v>
+      </c>
+      <c r="I9" t="n">
+        <v>15348644.75734568</v>
+      </c>
+      <c r="J9" t="n">
+        <v>27356236.08</v>
+      </c>
+      <c r="K9" t="n">
+        <v>28597259</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4885687.32</v>
+      </c>
+      <c r="M9" t="n">
+        <v>6872938.37913241</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2157709.42</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>1265375</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>-2639467.669999987</v>
+      </c>
+      <c r="S9" t="n">
+        <v>-1960946.43513241</v>
+      </c>
+      <c r="T9" t="n">
+        <v>-2476148</v>
+      </c>
+      <c r="U9" t="n">
+        <v>-2308110.319576854</v>
+      </c>
+      <c r="V9" t="n">
+        <v>162138200.08</v>
+      </c>
+      <c r="W9" t="n">
+        <v>192827759.600357</v>
+      </c>
+      <c r="X9" t="n">
+        <v>22237920.13</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>40971355.81690125</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>83238334.97</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>86895985.01353751</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>55622267.49000001</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>65020418.76991829</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dec-25</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>92056924.37999998</v>
+      </c>
+      <c r="C10" t="n">
+        <v>105112539.7619839</v>
+      </c>
+      <c r="D10" t="n">
+        <v>13669721.21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>24118315</v>
+      </c>
+      <c r="F10" t="n">
+        <v>53126006.13</v>
+      </c>
+      <c r="G10" t="n">
+        <v>64564850.52355281</v>
+      </c>
+      <c r="H10" t="n">
+        <v>9149765.82</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8733145.425684026</v>
+      </c>
+      <c r="J10" t="n">
+        <v>26941579.35</v>
+      </c>
+      <c r="K10" t="n">
+        <v>28975873</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5015843.060000001</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7145591.801489527</v>
+      </c>
+      <c r="N10" t="n">
+        <v>53778662.25</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>45087125</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-2037195.75999999</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-1983866.857489527</v>
+      </c>
+      <c r="T10" t="n">
+        <v>-2653712</v>
+      </c>
+      <c r="U10" t="n">
+        <v>-2331030.741933972</v>
+      </c>
+      <c r="V10" t="n">
+        <v>223865976.35</v>
+      </c>
+      <c r="W10" t="n">
+        <v>198731718.3280472</v>
+      </c>
+      <c r="X10" t="n">
+        <v>70268743.09</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>38137896.48523958</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>85821328.38999999</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>87502690.83408965</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>67899678.31999999</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>73151131.00871794</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>89570651.43000001</v>
+      </c>
+      <c r="C11" t="n">
+        <v>94892293.2192031</v>
+      </c>
+      <c r="D11" t="n">
+        <v>12704569.97</v>
+      </c>
+      <c r="E11" t="n">
+        <v>14100869.41</v>
+      </c>
+      <c r="F11" t="n">
+        <v>45833455.48</v>
+      </c>
+      <c r="G11" t="n">
+        <v>55775449.37978129</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5159112.889999998</v>
+      </c>
+      <c r="I11" t="n">
+        <v>8740611.206033947</v>
+      </c>
+      <c r="J11" t="n">
+        <v>26995058.56189249</v>
+      </c>
+      <c r="K11" t="n">
+        <v>29393218</v>
+      </c>
+      <c r="L11" t="n">
+        <v>5063916.859999999</v>
+      </c>
+      <c r="M11" t="n">
+        <v>7317661.119463768</v>
+      </c>
+      <c r="N11" t="n">
+        <v>29378388.9</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>24393875</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>-2351353.810000002</v>
+      </c>
+      <c r="S11" t="n">
+        <v>-1996431.175463768</v>
+      </c>
+      <c r="T11" t="n">
+        <v>-2773000</v>
+      </c>
+      <c r="U11" t="n">
+        <v>-2343595.059908213</v>
+      </c>
+      <c r="V11" t="n">
+        <v>189426200.5618925</v>
+      </c>
+      <c r="W11" t="n">
+        <v>181170857.5901873</v>
+      </c>
+      <c r="X11" t="n">
+        <v>44548474.72</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>28955637.27558951</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>65462556.84424999</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>81283075.27646777</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>79538114.5476425</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>70992145.03813002</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>86627198.53</v>
+      </c>
+      <c r="C12" t="n">
+        <v>96008362.93721315</v>
+      </c>
+      <c r="D12" t="n">
+        <v>12420253.18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>18468843.41</v>
+      </c>
+      <c r="F12" t="n">
+        <v>49594614.91</v>
+      </c>
+      <c r="G12" t="n">
+        <v>52209344.05719531</v>
+      </c>
+      <c r="H12" t="n">
+        <v>4697652.45</v>
+      </c>
+      <c r="I12" t="n">
+        <v>3764030.682719573</v>
+      </c>
+      <c r="J12" t="n">
+        <v>27244862.09</v>
+      </c>
+      <c r="K12" t="n">
+        <v>29880629</v>
+      </c>
+      <c r="L12" t="n">
+        <v>10988379.38</v>
+      </c>
+      <c r="M12" t="n">
+        <v>7495389.334991091</v>
+      </c>
+      <c r="N12" t="n">
+        <v>53371865.19</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>44301206.73</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-810386.6299999952</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-2004757.390991091</v>
+      </c>
+      <c r="T12" t="n">
+        <v>-905000</v>
+      </c>
+      <c r="U12" t="n">
+        <v>-2351921.275435536</v>
+      </c>
+      <c r="V12" t="n">
+        <v>216028154.09</v>
+      </c>
+      <c r="W12" t="n">
+        <v>179252406.770084</v>
+      </c>
+      <c r="X12" t="n">
+        <v>71502491.73999999</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>28516432.75227513</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>66132145.10608834</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>81717722.67198595</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>78514328.51391169</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>69078251.34582293</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>108214511.69</v>
+      </c>
+      <c r="C13" t="n">
+        <v>94631079.54768565</v>
+      </c>
+      <c r="D13" t="n">
+        <v>13045142.61</v>
+      </c>
+      <c r="E13" t="n">
+        <v>17868311</v>
+      </c>
+      <c r="F13" t="n">
+        <v>82925659.89</v>
+      </c>
+      <c r="G13" t="n">
+        <v>66884533.84582798</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1836751.030000004</v>
+      </c>
+      <c r="I13" t="n">
+        <v>14313238.62119834</v>
+      </c>
+      <c r="J13" t="n">
+        <v>29642976.66</v>
+      </c>
+      <c r="K13" t="n">
+        <v>30155964</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4603785.73</v>
+      </c>
+      <c r="M13" t="n">
+        <v>7734181.205156771</v>
+      </c>
+      <c r="N13" t="n">
+        <v>908753.9300000001</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>243119.99</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-2103099.51000002</v>
+      </c>
+      <c r="S13" t="n">
+        <v>-2985901.491156771</v>
+      </c>
+      <c r="T13" t="n">
+        <v>-14457484.17</v>
+      </c>
+      <c r="U13" t="n">
+        <v>-2365427.145601215</v>
+      </c>
+      <c r="V13" t="n">
+        <v>219588802.66</v>
+      </c>
+      <c r="W13" t="n">
+        <v>199291615.1690235</v>
+      </c>
+      <c r="X13" t="n">
+        <v>5271315.190000005</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>40490394.2807539</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>111963280.11</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>86293632.73162086</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>107853458.94</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>72567588.15664874</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>91096868.77000003</v>
+      </c>
+      <c r="C14" t="n">
+        <v>80274532.4636035</v>
+      </c>
+      <c r="D14" t="n">
+        <v>14010859.5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>10442347.08371727</v>
+      </c>
+      <c r="F14" t="n">
+        <v>46030788.94</v>
+      </c>
+      <c r="G14" t="n">
+        <v>46530148.5645342</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2993618.490000005</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3881417.21134247</v>
+      </c>
+      <c r="J14" t="n">
+        <v>25447329.81</v>
+      </c>
+      <c r="K14" t="n">
+        <v>28894159.2091278</v>
+      </c>
+      <c r="L14" t="n">
+        <v>5052508.66</v>
+      </c>
+      <c r="M14" t="n">
+        <v>5142998.307669034</v>
+      </c>
+      <c r="N14" t="n">
+        <v>938594.01</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>217680.38</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-2000000</v>
+      </c>
+      <c r="S14" t="n">
+        <v>-2953301.1165</v>
+      </c>
+      <c r="T14" t="n">
+        <v>-1834298</v>
+      </c>
+      <c r="U14" t="n">
+        <v>-2217682.8665</v>
+      </c>
+      <c r="V14" t="n">
+        <v>161513581.53</v>
+      </c>
+      <c r="W14" t="n">
+        <v>153681628.0207655</v>
+      </c>
+      <c r="X14" t="n">
+        <v>20440369.03</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>17464854.98622877</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>70534458.91</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>78962885.94843617</v>
+      </c>
+      <c r="AB14" t="n">
+        <v>70625668.58000004</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>57308900.91610059</v>
       </c>
     </row>
   </sheetData>
@@ -3798,7 +3801,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Plan</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -3808,73 +3811,83 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Monthly_Fee_TTD</t>
+          <t>ARPU_Band_TTD</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Basic Voice</t>
+          <t>Very Low</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>45000</v>
-      </c>
-      <c r="C2" t="n">
-        <v>99</v>
+        <v>220000</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>&lt; $50</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Basic Data</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38000</v>
-      </c>
-      <c r="C3" t="n">
-        <v>149</v>
+        <v>185000</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>$50 - $100</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Standard Bundle</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22000</v>
-      </c>
-      <c r="C4" t="n">
-        <v>249</v>
+        <v>130000</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>$101 - $200</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Premium Bundle</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>399</v>
+        <v>60000</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>$201 - $400</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Very High</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8000</v>
-      </c>
-      <c r="C6" t="n">
-        <v>699</v>
+        <v>25000</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>&gt; $400</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WTTx donut: replace ARPU categories with plan type (Voice Only / Bundles / Data Only)
Added WTTx_Plans sheet to Excel — edit Subscribers column to update live data.
Height increased to 420px to match Postpaid. Colours: amber / purple / teal.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="6" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,9 +22,10 @@
     <sheet name="PnL_Breakdown" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Pre_ARPU_Cats" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="WTTx_ARPU_Cats" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="WTTx_Plans" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
 </file>
 
@@ -453,7 +454,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -653,7 +654,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1417,7 +1418,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1881,7 +1882,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2344,6 +2345,11 @@
   </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2369,20 +2375,20 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>180000</v>
+        <v>65000</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Basic Voice</t>
+          <t>Cheapo plan</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45000</v>
+        <v>33000</v>
       </c>
       <c r="C3" t="n">
         <v>99</v>
@@ -2391,11 +2397,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Basic Data</t>
+          <t>Basic Plan</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>38000</v>
+        <v>12000</v>
       </c>
       <c r="C4" t="n">
         <v>149</v>
@@ -2404,11 +2410,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Standard Bundle</t>
+          <t>Special Plan</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22000</v>
+        <v>4000</v>
       </c>
       <c r="C5" t="n">
         <v>249</v>
@@ -2417,11 +2423,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Premium Bundle</t>
+          <t>Rich People plan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15000</v>
+        <v>2500</v>
       </c>
       <c r="C6" t="n">
         <v>399</v>
@@ -2430,11 +2436,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Enterprise</t>
+          <t>Super Rich People</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8000</v>
+        <v>150</v>
       </c>
       <c r="C7" t="n">
         <v>699</v>
@@ -2452,7 +2458,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4001,6 +4007,62 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Subscribers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Voice Only</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bundles</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Data Only</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>62000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4008,7 +4070,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4452,7 +4514,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4578,7 +4640,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F145"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -7882,7 +7944,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -8197,16 +8259,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H79"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7.08984375" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.08984375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="11.81640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="12.6328125" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="10.36328125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="9.54296875" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="11.81640625" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="14.81640625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="7.140625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12.5703125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.42578125" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="9.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="11.85546875" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10387,7 +10449,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I92"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -13157,7 +13219,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -13203,7 +13265,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Data: add Apr-26 row to Cash_CAPEX sheet
Cash Balance: 220,070,000 | FCF: -128,887,000 | Net Debt: 3,228,914,000

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSTT_Board_Data.xlsx
+++ b/TSTT_Board_Data.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="3" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,14 +21,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PnL_Breakdown" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterate="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,7 +37,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <sz val="8"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -58,10 +66,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -74,7 +91,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -696,7 +713,6 @@
       <c r="C2" t="n">
         <v>820297.73</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -724,7 +740,6 @@
       <c r="C3" t="n">
         <v>29407.38</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -752,7 +767,6 @@
       <c r="C4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -780,7 +794,6 @@
       <c r="C5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -808,7 +821,6 @@
       <c r="C6" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -836,7 +848,6 @@
       <c r="C7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -864,7 +875,6 @@
       <c r="C8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0</v>
       </c>
@@ -892,7 +902,6 @@
       <c r="C9" t="n">
         <v>1008044</v>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -920,7 +929,6 @@
       <c r="C10" t="n">
         <v>-59481.12</v>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0</v>
       </c>
@@ -948,7 +956,6 @@
       <c r="C11" t="n">
         <v>450000</v>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -976,7 +983,6 @@
       <c r="C12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>0</v>
       </c>
@@ -1004,7 +1010,6 @@
       <c r="C13" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -1032,7 +1037,6 @@
       <c r="C14" t="n">
         <v>543.16</v>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>0</v>
       </c>
@@ -1060,7 +1064,6 @@
       <c r="C15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>0</v>
       </c>
@@ -1088,7 +1091,6 @@
       <c r="C16" t="n">
         <v>819122.22</v>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>0</v>
       </c>
@@ -1116,7 +1118,6 @@
       <c r="C17" t="n">
         <v>29407.78</v>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>0</v>
       </c>
@@ -1144,7 +1145,6 @@
       <c r="C18" t="n">
         <v>0</v>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
         <v>0</v>
       </c>
@@ -1172,7 +1172,6 @@
       <c r="C19" t="n">
         <v>0</v>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>0</v>
       </c>
@@ -1200,7 +1199,6 @@
       <c r="C20" t="n">
         <v>0</v>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>0</v>
       </c>
@@ -1228,7 +1226,6 @@
       <c r="C21" t="n">
         <v>937.6</v>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>0</v>
       </c>
@@ -1256,7 +1253,6 @@
       <c r="C22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>0</v>
       </c>
@@ -1284,7 +1280,6 @@
       <c r="C23" t="n">
         <v>810855.89</v>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>0</v>
       </c>
@@ -1312,7 +1307,6 @@
       <c r="C24" t="n">
         <v>0</v>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>0</v>
       </c>
@@ -1340,7 +1334,6 @@
       <c r="C25" t="n">
         <v>0</v>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -1368,7 +1361,6 @@
       <c r="C26" t="n">
         <v>0</v>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>0</v>
       </c>
@@ -1396,7 +1388,6 @@
       <c r="C27" t="n">
         <v>0</v>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>0</v>
       </c>
@@ -1424,7 +1415,6 @@
       <c r="C28" t="n">
         <v>1010.64</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>0</v>
       </c>
@@ -1452,7 +1442,6 @@
       <c r="C29" t="n">
         <v>0</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>0</v>
       </c>
@@ -1480,7 +1469,6 @@
       <c r="C30" t="n">
         <v>819188.89</v>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>0</v>
       </c>
@@ -1508,7 +1496,6 @@
       <c r="C31" t="n">
         <v>0</v>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>0</v>
       </c>
@@ -1536,7 +1523,6 @@
       <c r="C32" t="n">
         <v>0</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>0</v>
       </c>
@@ -1564,7 +1550,6 @@
       <c r="C33" t="n">
         <v>0</v>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>0</v>
       </c>
@@ -1592,7 +1577,6 @@
       <c r="C34" t="n">
         <v>355555.6</v>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>0</v>
       </c>
@@ -1620,7 +1604,6 @@
       <c r="C35" t="n">
         <v>463.7</v>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0</v>
       </c>
@@ -1648,7 +1631,6 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>0</v>
       </c>
@@ -1676,7 +1658,6 @@
       <c r="C37" t="n">
         <v>859566.67</v>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0</v>
       </c>
@@ -1704,7 +1685,6 @@
       <c r="C38" t="n">
         <v>-17847.78</v>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>0</v>
       </c>
@@ -1732,7 +1712,6 @@
       <c r="C39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>0</v>
       </c>
@@ -1760,7 +1739,6 @@
       <c r="C40" t="n">
         <v>0</v>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>0</v>
       </c>
@@ -1788,7 +1766,6 @@
       <c r="C41" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -1816,7 +1793,6 @@
       <c r="C42" t="n">
         <v>674.72</v>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -1844,7 +1820,6 @@
       <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>0</v>
       </c>
@@ -1872,7 +1847,6 @@
       <c r="C44" t="n">
         <v>820811.11</v>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>0</v>
       </c>
@@ -1900,7 +1874,6 @@
       <c r="C45" t="n">
         <v>0</v>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>0</v>
       </c>
@@ -1928,7 +1901,6 @@
       <c r="C46" t="n">
         <v>0</v>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>0</v>
       </c>
@@ -1956,7 +1928,6 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>0</v>
       </c>
@@ -1984,7 +1955,6 @@
       <c r="C48" t="n">
         <v>258871.4</v>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0</v>
       </c>
@@ -2012,7 +1982,6 @@
       <c r="C49" t="n">
         <v>0</v>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0</v>
       </c>
@@ -2040,7 +2009,6 @@
       <c r="C50" t="n">
         <v>0</v>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>0</v>
       </c>
@@ -2068,7 +2036,6 @@
       <c r="C51" t="n">
         <v>819655.5600000001</v>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>0</v>
       </c>
@@ -2096,7 +2063,6 @@
       <c r="C52" t="n">
         <v>-11560</v>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>0</v>
       </c>
@@ -2124,7 +2090,6 @@
       <c r="C53" t="n">
         <v>0</v>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
         <v>0</v>
       </c>
@@ -2152,7 +2117,6 @@
       <c r="C54" t="n">
         <v>0</v>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>0</v>
       </c>
@@ -2180,7 +2144,6 @@
       <c r="C55" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0</v>
       </c>
@@ -2208,7 +2171,6 @@
       <c r="C56" t="n">
         <v>724.96</v>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>0</v>
       </c>
@@ -2236,7 +2198,6 @@
       <c r="C57" t="n">
         <v>1260000</v>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>0</v>
       </c>
@@ -2264,7 +2225,6 @@
       <c r="C58" t="n">
         <v>874238.89</v>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>0</v>
       </c>
@@ -2292,7 +2252,6 @@
       <c r="C59" t="n">
         <v>0</v>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>0</v>
       </c>
@@ -2320,7 +2279,6 @@
       <c r="C60" t="n">
         <v>0</v>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>0</v>
       </c>
@@ -2348,7 +2306,6 @@
       <c r="C61" t="n">
         <v>0</v>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>0</v>
       </c>
@@ -2376,7 +2333,6 @@
       <c r="C62" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>0</v>
       </c>
@@ -2404,7 +2360,6 @@
       <c r="C63" t="n">
         <v>534.46</v>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>0</v>
       </c>
@@ -2432,7 +2387,6 @@
       <c r="C64" t="n">
         <v>52815000</v>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>0</v>
       </c>
@@ -2460,7 +2414,6 @@
       <c r="C65" t="n">
         <v>819500</v>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0</v>
       </c>
@@ -2488,7 +2441,6 @@
       <c r="C66" t="n">
         <v>0</v>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>0</v>
       </c>
@@ -2516,7 +2468,6 @@
       <c r="C67" t="n">
         <v>0</v>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>0</v>
       </c>
@@ -2544,7 +2495,6 @@
       <c r="C68" t="n">
         <v>0</v>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>0</v>
       </c>
@@ -2572,7 +2522,6 @@
       <c r="C69" t="n">
         <v>88888.89999999999</v>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>0</v>
       </c>
@@ -2600,7 +2549,6 @@
       <c r="C70" t="n">
         <v>0</v>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>0</v>
       </c>
@@ -2628,7 +2576,6 @@
       <c r="C71" t="n">
         <v>28470000</v>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>0</v>
       </c>
@@ -2656,7 +2603,6 @@
       <c r="C72" t="n">
         <v>825611.11</v>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>0</v>
       </c>
@@ -2684,7 +2630,6 @@
       <c r="C73" t="n">
         <v>0</v>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>0</v>
       </c>
@@ -2712,7 +2657,6 @@
       <c r="C74" t="n">
         <v>0</v>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="n">
         <v>0</v>
       </c>
@@ -2740,7 +2684,6 @@
       <c r="C75" t="n">
         <v>0</v>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
         <v>0</v>
       </c>
@@ -2768,7 +2711,6 @@
       <c r="C76" t="n">
         <v>88368.07999999999</v>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>0</v>
       </c>
@@ -2796,7 +2738,6 @@
       <c r="C77" t="n">
         <v>2886</v>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>0</v>
       </c>
@@ -2824,7 +2765,6 @@
       <c r="C78" t="n">
         <v>52455000</v>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>0</v>
       </c>
@@ -2852,7 +2792,6 @@
       <c r="C79" t="n">
         <v>818766.67</v>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>0</v>
       </c>
@@ -2880,7 +2819,6 @@
       <c r="C80" t="n">
         <v>0</v>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
         <v>0</v>
       </c>
@@ -2908,7 +2846,6 @@
       <c r="C81" t="n">
         <v>0</v>
       </c>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="n">
         <v>0</v>
       </c>
@@ -2936,7 +2873,6 @@
       <c r="C82" t="n">
         <v>0</v>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
         <v>0</v>
       </c>
@@ -2964,7 +2900,6 @@
       <c r="C83" t="n">
         <v>89807.25999999999</v>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
         <v>0</v>
       </c>
@@ -2992,7 +2927,6 @@
       <c r="C84" t="n">
         <v>180</v>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
         <v>0</v>
       </c>
@@ -3020,7 +2954,6 @@
       <c r="C85" t="n">
         <v>0</v>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="n">
         <v>0</v>
       </c>
@@ -3314,14 +3247,12 @@
       <c r="B2" t="n">
         <v>25447329.81</v>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>20394821.15</v>
       </c>
       <c r="E2" t="n">
         <v>9951562.490000002</v>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>3232985.520000002</v>
       </c>
@@ -3341,14 +3272,12 @@
       <c r="B3" t="n">
         <v>26113220.11</v>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>21340447.63</v>
       </c>
       <c r="E3" t="n">
         <v>11267071.63</v>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>4198005.439999999</v>
       </c>
@@ -3368,14 +3297,12 @@
       <c r="B4" t="n">
         <v>26264263.11999999</v>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>21395764.34</v>
       </c>
       <c r="E4" t="n">
         <v>10980632.72</v>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>2739683.559999995</v>
       </c>
@@ -3395,14 +3322,12 @@
       <c r="B5" t="n">
         <v>26813033.17</v>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>21924533.09</v>
       </c>
       <c r="E5" t="n">
         <v>12059566.26999999</v>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>7074220.709999993</v>
       </c>
@@ -3422,14 +3347,12 @@
       <c r="B6" t="n">
         <v>26736564.21</v>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>21898090.24</v>
       </c>
       <c r="E6" t="n">
         <v>11190450.52334339</v>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>4567268.193343389</v>
       </c>
@@ -3449,14 +3372,12 @@
       <c r="B7" t="n">
         <v>26178595.18</v>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>21993768.09</v>
       </c>
       <c r="E7" t="n">
         <v>11975663.99</v>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>4800162.980000002</v>
       </c>
@@ -3476,14 +3397,12 @@
       <c r="B8" t="n">
         <v>27643427.7</v>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>22911774.08</v>
       </c>
       <c r="E8" t="n">
         <v>10392674.96</v>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>3318782.899999993</v>
       </c>
@@ -3503,14 +3422,12 @@
       <c r="B9" t="n">
         <v>27356236.08</v>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>22470548.76</v>
       </c>
       <c r="E9" t="n">
         <v>11822575.61</v>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>3928525.235190003</v>
       </c>
@@ -3530,14 +3447,12 @@
       <c r="B10" t="n">
         <v>26941579.35</v>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
         <v>21925736.29</v>
       </c>
       <c r="E10" t="n">
         <v>11253973.75</v>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>3568403.039999997</v>
       </c>
@@ -3557,14 +3472,12 @@
       <c r="B11" t="n">
         <v>26995058.56189249</v>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
         <v>21931141.70189249</v>
       </c>
       <c r="E11" t="n">
         <v>11456168.96764249</v>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>6550708.337642494</v>
       </c>
@@ -3584,14 +3497,12 @@
       <c r="B12" t="n">
         <v>27244862.09</v>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
         <v>16256482.71</v>
       </c>
       <c r="E12" t="n">
         <v>14080874.28391166</v>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>6770120.643911664</v>
       </c>
@@ -3611,14 +3522,12 @@
       <c r="B13" t="n">
         <v>29642976.66</v>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="n">
         <v>25039190.93</v>
       </c>
       <c r="E13" t="n">
         <v>10696196.07</v>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>2715600.420000001</v>
       </c>
@@ -3647,7 +3556,6 @@
       <c r="E14" t="n">
         <v>12554599.36999999</v>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>4614266.819999992</v>
       </c>
@@ -5553,9 +5461,6 @@
       <c r="E2" t="n">
         <v>0.437273868308603</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>159174265.27</v>
       </c>
@@ -5584,9 +5489,6 @@
       <c r="E3" t="n">
         <v>0.4073280166649205</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>171115783.94</v>
       </c>
@@ -5615,9 +5517,6 @@
       <c r="E4" t="n">
         <v>0.5025764629697752</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
         <v>156481421.44</v>
       </c>
@@ -5646,9 +5545,6 @@
       <c r="E5" t="n">
         <v>0.4666812777131023</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
         <v>189874779.76</v>
       </c>
@@ -5677,9 +5573,6 @@
       <c r="E6" t="n">
         <v>0.5185481722298699</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>166311231.95</v>
       </c>
@@ -5708,9 +5601,6 @@
       <c r="E7" t="n">
         <v>0.3232868088131722</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
         <v>166133918.48</v>
       </c>
@@ -5739,9 +5629,6 @@
       <c r="E8" t="n">
         <v>0.5353363116736716</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>162482252.18</v>
       </c>
@@ -5770,9 +5657,6 @@
       <c r="E9" t="n">
         <v>0.3430546747315292</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
         <v>164022306.72</v>
       </c>
@@ -5801,9 +5685,6 @@
       <c r="E10" t="n">
         <v>0.3033050373579022</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>162105315.02</v>
       </c>
@@ -5832,9 +5713,6 @@
       <c r="E11" t="n">
         <v>0.4198897212302714</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>157291107.71</v>
       </c>
@@ -5863,9 +5741,6 @@
       <c r="E12" t="n">
         <v>0.3634448891379299</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>153534324.86</v>
       </c>
@@ -5894,9 +5769,6 @@
       <c r="E13" t="n">
         <v>0.4315246523599764</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
         <v>49698939.2</v>
       </c>
@@ -6083,6 +5955,10 @@
   </sheetPr>
   <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -6130,7 +6006,6 @@
       <c r="C2" t="n">
         <v>19177303.91</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -6152,7 +6027,6 @@
       <c r="C3" t="n">
         <v>22798838.08</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -6171,8 +6045,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -6194,7 +6066,6 @@
       <c r="C5" t="n">
         <v>25999329.58</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -6216,7 +6087,6 @@
       <c r="C6" t="n">
         <v>2558987.34</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -6235,8 +6105,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -6258,7 +6126,6 @@
       <c r="C8" t="n">
         <v>16866294.79496403</v>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0</v>
       </c>
@@ -6280,7 +6147,6 @@
       <c r="C9" t="n">
         <v>24192810.22</v>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -6299,8 +6165,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0</v>
       </c>
@@ -6322,7 +6186,6 @@
       <c r="C11" t="n">
         <v>32324520.08000001</v>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -6344,7 +6207,6 @@
       <c r="C12" t="n">
         <v>2426943.79</v>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>0</v>
       </c>
@@ -6363,8 +6225,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -6386,7 +6246,6 @@
       <c r="C14" t="n">
         <v>18338058.404</v>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>0</v>
       </c>
@@ -6408,7 +6267,6 @@
       <c r="C15" t="n">
         <v>19811291.25</v>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>0</v>
       </c>
@@ -6427,8 +6285,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>0</v>
       </c>
@@ -6450,7 +6306,6 @@
       <c r="C17" t="n">
         <v>19931554.91</v>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>0</v>
       </c>
@@ -6472,7 +6327,6 @@
       <c r="C18" t="n">
         <v>3058121.92</v>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
         <v>0</v>
       </c>
@@ -6491,8 +6345,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>0</v>
       </c>
@@ -6514,7 +6366,6 @@
       <c r="C20" t="n">
         <v>20186695.95740462</v>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>0</v>
       </c>
@@ -6536,7 +6387,6 @@
       <c r="C21" t="n">
         <v>18958609.92</v>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>0</v>
       </c>
@@ -6555,8 +6405,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>0</v>
       </c>
@@ -6578,7 +6426,6 @@
       <c r="C23" t="n">
         <v>27432588.48</v>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>0</v>
       </c>
@@ -6600,7 +6447,6 @@
       <c r="C24" t="n">
         <v>2770972</v>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>0</v>
       </c>
@@ -6619,8 +6465,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -6642,7 +6486,6 @@
       <c r="C26" t="n">
         <v>17208083.38</v>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>0</v>
       </c>
@@ -6664,7 +6507,6 @@
       <c r="C27" t="n">
         <v>20792286.49</v>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>0</v>
       </c>
@@ -6683,8 +6525,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>0</v>
       </c>
@@ -6706,7 +6546,6 @@
       <c r="C29" t="n">
         <v>20303813.92</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>0</v>
       </c>
@@ -6728,7 +6567,6 @@
       <c r="C30" t="n">
         <v>-1164889.453343391</v>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>0</v>
       </c>
@@ -6747,8 +6585,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>0</v>
       </c>
@@ -6770,7 +6606,6 @@
       <c r="C32" t="n">
         <v>19235316.19</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>0</v>
       </c>
@@ -6792,7 +6627,6 @@
       <c r="C33" t="n">
         <v>27652891.77</v>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>0</v>
       </c>
@@ -6811,8 +6645,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>0</v>
       </c>
@@ -6834,7 +6666,6 @@
       <c r="C35" t="n">
         <v>39223866.20000001</v>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0</v>
       </c>
@@ -6856,7 +6687,6 @@
       <c r="C36" t="n">
         <v>2277498.62</v>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>0</v>
       </c>
@@ -6875,8 +6705,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0</v>
       </c>
@@ -6898,7 +6726,6 @@
       <c r="C38" t="n">
         <v>19039407.04</v>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>0</v>
       </c>
@@ -6920,7 +6747,6 @@
       <c r="C39" t="n">
         <v>22303868.43000001</v>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>0</v>
       </c>
@@ -6939,8 +6765,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>0</v>
       </c>
@@ -6962,7 +6786,6 @@
       <c r="C41" t="n">
         <v>12586832.32999999</v>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -6984,7 +6807,6 @@
       <c r="C42" t="n">
         <v>3743552.41</v>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -7003,8 +6825,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>0</v>
       </c>
@@ -7026,7 +6846,6 @@
       <c r="C44" t="n">
         <v>26809267.37</v>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>0</v>
       </c>
@@ -7048,7 +6867,6 @@
       <c r="C45" t="n">
         <v>23590475.35</v>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>0</v>
       </c>
@@ -7067,8 +6885,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>0</v>
       </c>
@@ -7090,7 +6906,6 @@
       <c r="C47" t="n">
         <v>28556489.68</v>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>0</v>
       </c>
@@ -7112,7 +6927,6 @@
       <c r="C48" t="n">
         <v>4282102.569999999</v>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0</v>
       </c>
@@ -7131,8 +6945,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0</v>
       </c>
@@ -7154,7 +6966,6 @@
       <c r="C50" t="n">
         <v>18508183.54</v>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>0</v>
       </c>
@@ -7176,7 +6987,6 @@
       <c r="C51" t="n">
         <v>15931690.15</v>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>0</v>
       </c>
@@ -7195,8 +7005,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>0</v>
       </c>
@@ -7218,7 +7026,6 @@
       <c r="C53" t="n">
         <v>53094640.03999998</v>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
         <v>0</v>
       </c>
@@ -7240,7 +7047,6 @@
       <c r="C54" t="n">
         <v>-1713185.34</v>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>0</v>
       </c>
@@ -7259,8 +7065,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0</v>
       </c>
@@ -7282,7 +7086,6 @@
       <c r="C56" t="n">
         <v>20903874.39</v>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>0</v>
       </c>
@@ -7304,7 +7107,6 @@
       <c r="C57" t="n">
         <v>19114631.63</v>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>0</v>
       </c>
@@ -7323,8 +7125,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>0</v>
       </c>
@@ -7346,7 +7146,6 @@
       <c r="C59" t="n">
         <v>18510872.70424999</v>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>0</v>
       </c>
@@ -7368,7 +7167,6 @@
       <c r="C60" t="n">
         <v>6933178.119999999</v>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>0</v>
       </c>
@@ -7387,8 +7185,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>0</v>
       </c>
@@ -7410,7 +7206,6 @@
       <c r="C62" t="n">
         <v>19632643.9</v>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>0</v>
       </c>
@@ -7432,7 +7227,6 @@
       <c r="C63" t="n">
         <v>13671833.22</v>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>0</v>
       </c>
@@ -7451,8 +7245,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>0</v>
       </c>
@@ -7474,7 +7266,6 @@
       <c r="C65" t="n">
         <v>31766772.76608834</v>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0</v>
       </c>
@@ -7496,7 +7287,6 @@
       <c r="C66" t="n">
         <v>1060895.22</v>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>0</v>
       </c>
@@ -7515,8 +7305,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>0</v>
       </c>
@@ -7538,7 +7326,6 @@
       <c r="C68" t="n">
         <v>20770066.68</v>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>0</v>
       </c>
@@ -7560,7 +7347,6 @@
       <c r="C69" t="n">
         <v>30469543.92</v>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>0</v>
       </c>
@@ -7579,8 +7365,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>0</v>
       </c>
@@ -7602,7 +7386,6 @@
       <c r="C71" t="n">
         <v>23040621.34000001</v>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>0</v>
       </c>
@@ -7624,7 +7407,6 @@
       <c r="C72" t="n">
         <v>31273106.29</v>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>0</v>
       </c>
@@ -7643,8 +7425,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>0</v>
       </c>
@@ -7711,9 +7491,11 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="n">
+        <v>2237645.1</v>
+      </c>
       <c r="D76" t="n">
-        <v>13975641.44476191</v>
+        <v>4825993.819165427</v>
       </c>
       <c r="E76" t="n">
         <v>0</v>
@@ -7734,10 +7516,10 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>16729457.01000001</v>
+        <v>13488346.06</v>
       </c>
       <c r="D77" t="n">
-        <v>17641296.31599329</v>
+        <v>23155080.47678529</v>
       </c>
       <c r="E77" t="n">
         <v>0</v>
@@ -7781,7 +7563,9 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
+      <c r="C79" t="n">
+        <v>1003465.85</v>
+      </c>
       <c r="D79" t="n">
         <v>2248453.405862648</v>
       </c>
@@ -7803,7 +7587,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="n">
         <v>22591612.33270326</v>
       </c>
@@ -7825,7 +7608,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="n">
         <v>23147297.86274611</v>
       </c>
@@ -7847,7 +7629,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="n">
         <v>14332013.6352381</v>
       </c>
@@ -7869,7 +7650,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="n">
         <v>17646306.05536446</v>
       </c>
@@ -7891,7 +7671,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="n">
         <v>3168047.030440447</v>
       </c>
@@ -7913,7 +7692,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="n">
         <v>3241953.232895536</v>
       </c>
@@ -7935,7 +7713,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="n">
         <v>22522911.54131892</v>
       </c>
@@ -7957,7 +7734,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="n">
         <v>23871463.00056273</v>
       </c>
@@ -7979,7 +7755,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="n">
         <v>17173048.7052381</v>
       </c>
@@ -8001,7 +7776,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="n">
         <v>19474521.73444509</v>
       </c>
@@ -8023,7 +7797,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="n">
         <v>3294321.145640145</v>
       </c>
@@ -8045,7 +7818,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="n">
         <v>5201350.327907625</v>
       </c>
@@ -8067,7 +7839,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="n">
         <v>22657637.09599318</v>
       </c>
@@ -8089,7 +7860,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="n">
         <v>22771503.68704942</v>
       </c>
@@ -8111,7 +7881,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="n">
         <v>15169612.6352381</v>
       </c>
@@ -8133,7 +7902,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="n">
         <v>110707370.9709836</v>
       </c>
@@ -8155,7 +7923,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="n">
         <v>3725840.471526688</v>
       </c>
@@ -8177,7 +7944,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="n">
         <v>2842128.722017645</v>
       </c>
@@ -8199,7 +7965,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="n">
         <v>22986653.2146912</v>
       </c>
@@ -8221,7 +7986,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="n">
         <v>23101642.49688293</v>
       </c>
@@ -8243,7 +8007,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="n">
         <v>14093039.44476191</v>
       </c>
@@ -8265,7 +8028,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="n">
         <v>18031437.18467504</v>
       </c>
@@ -8287,7 +8049,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="n">
         <v>3794023.364505047</v>
       </c>
@@ -8309,7 +8070,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="n">
         <v>4722333.82309229</v>
       </c>
@@ -8331,7 +8091,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="n">
         <v>22449175.76470205</v>
       </c>
@@ -8353,7 +8112,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="n">
         <v>24163742.91004469</v>
       </c>
@@ -8375,7 +8133,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
         <v>14907237.44476191</v>
       </c>
@@ -8397,7 +8154,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="n">
         <v>18899174.40615667</v>
       </c>
@@ -8419,7 +8175,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="n">
         <v>3839645.503585657</v>
       </c>
@@ -8441,7 +8196,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="n">
         <v>2740233.653965407</v>
       </c>
@@ -8463,7 +8217,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="n">
         <v>22648513.31474198</v>
       </c>
@@ -8485,7 +8238,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
       <c r="D111" t="n">
         <v>23504509.50771018</v>
       </c>
@@ -8507,7 +8259,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
         <v>12840482.78476191</v>
       </c>
@@ -8529,7 +8280,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr"/>
       <c r="D113" t="n">
         <v>20078615.34753704</v>
       </c>
@@ -8551,7 +8301,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" t="n">
         <v>3216356.398978495</v>
       </c>
@@ -8573,7 +8322,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr"/>
       <c r="D115" t="n">
         <v>2060918.427395666</v>
       </c>
@@ -8595,7 +8343,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="n">
         <v>22674603.91006402</v>
       </c>
@@ -8617,7 +8364,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="n">
         <v>23892351.16330291</v>
       </c>
@@ -8639,7 +8385,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr"/>
       <c r="D118" t="n">
         <v>12530391.5047619</v>
       </c>
@@ -8661,7 +8406,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="n">
         <v>17771069.28279239</v>
       </c>
@@ -8683,7 +8427,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="n">
         <v>3247746.489788108</v>
       </c>
@@ -8705,7 +8448,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="n">
         <v>3116406.813288246</v>
       </c>
@@ -8727,7 +8469,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="n">
         <v>23470015.95171413</v>
       </c>
@@ -8749,7 +8490,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" t="n">
         <v>24792477.47404118</v>
       </c>
@@ -8771,7 +8511,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="n">
         <v>14611795.18476191</v>
       </c>
@@ -8793,7 +8532,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="n">
         <v>18760745.56039985</v>
       </c>
@@ -8815,7 +8553,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="n">
         <v>3409858.838336057</v>
       </c>
@@ -8837,7 +8574,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="n">
         <v>4505334.575696514</v>
       </c>
@@ -8859,7 +8595,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="n">
         <v>22621936.55925866</v>
       </c>
@@ -8881,7 +8616,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="n">
         <v>23642786.40061948</v>
       </c>
@@ -8903,7 +8637,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr"/>
       <c r="D130" t="n">
         <v>12016926.99428571</v>
       </c>
@@ -8925,7 +8658,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="n">
         <v>17390186.84683962</v>
       </c>
@@ -8947,7 +8679,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="n">
         <v>3456084.406932943</v>
       </c>
@@ -8969,7 +8700,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="n">
         <v>3683298.36296571</v>
       </c>
@@ -8991,7 +8721,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="n">
         <v>22769135.05253517</v>
       </c>
@@ -9013,7 +8742,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
         <v>24158478.22805225</v>
       </c>
@@ -9035,7 +8763,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
         <v>12033698.99428571</v>
       </c>
@@ -9057,7 +8784,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="n">
         <v>17379633.51987506</v>
       </c>
@@ -9079,7 +8805,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr"/>
       <c r="D138" t="n">
         <v>3477804.401558435</v>
       </c>
@@ -9101,7 +8826,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
         <v>3293437.961245519</v>
       </c>
@@ -9123,7 +8847,6 @@
           <t>Personnel</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
         <v>74718831.42457715</v>
       </c>
@@ -9145,7 +8868,6 @@
           <t>Maintenance</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
         <v>27331633.67587252</v>
       </c>
@@ -9167,7 +8889,6 @@
           <t>Consultancy &amp; Professional Fees</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr"/>
       <c r="D142" t="n">
         <v>11529703.99428571</v>
       </c>
@@ -9189,7 +8910,6 @@
           <t>Other Operating Expenses</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr"/>
       <c r="D143" t="n">
         <v>106066711.6235541</v>
       </c>
@@ -9211,7 +8931,6 @@
           <t>Bad Debt</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
         <v>3598284.039392758</v>
       </c>
@@ -9233,7 +8952,6 @@
           <t>Advertising &amp; PR</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
         <v>1977959.772256132</v>
       </c>
@@ -9255,8 +8973,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="13.140625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="13.42578125" bestFit="1" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -9316,7 +9042,6 @@
       <c r="F2" t="n">
         <v>10792000</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9339,7 +9064,6 @@
       <c r="F3" t="n">
         <v>23912000</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9362,7 +9086,6 @@
       <c r="F4" t="n">
         <v>14219000</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9385,7 +9108,6 @@
       <c r="F5" t="n">
         <v>24791000</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -9408,7 +9130,6 @@
       <c r="F6" t="n">
         <v>8949000</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -9431,7 +9152,6 @@
       <c r="F7" t="n">
         <v>18089000</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9454,7 +9174,6 @@
       <c r="F8" t="n">
         <v>31759000</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9477,7 +9196,6 @@
       <c r="F9" t="n">
         <v>44506000</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9500,7 +9218,6 @@
       <c r="F10" t="n">
         <v>22803000</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9523,7 +9240,6 @@
       <c r="F11" t="n">
         <v>35050000</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9546,7 +9262,6 @@
       <c r="F12" t="n">
         <v>13194000</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9569,7 +9284,28 @@
       <c r="F13" t="n">
         <v>49962000</v>
       </c>
-      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apr-26</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>220070000</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3228914000</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-128887000</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9584,6 +9320,15 @@
   </sheetPr>
   <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.140625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="10" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="15.85546875" bestFit="1" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -9641,7 +9386,6 @@
       <c r="C2" t="n">
         <v>31193266.66000001</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>104426</v>
       </c>
@@ -9669,7 +9413,6 @@
       <c r="C3" t="n">
         <v>34532303.34</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>418249</v>
       </c>
@@ -9697,7 +9440,6 @@
       <c r="C4" t="n">
         <v>16493687.29</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>103490</v>
       </c>
@@ -9722,8 +9464,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -9748,8 +9488,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -9777,7 +9515,6 @@
       <c r="C7" t="n">
         <v>10159919.31000002</v>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -9805,7 +9542,6 @@
       <c r="C8" t="n">
         <v>32261590.82000001</v>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>105314</v>
       </c>
@@ -9833,7 +9569,6 @@
       <c r="C9" t="n">
         <v>31947105.5</v>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>408145</v>
       </c>
@@ -9861,7 +9596,6 @@
       <c r="C10" t="n">
         <v>16471191.17</v>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>104166</v>
       </c>
@@ -9886,8 +9620,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -9912,8 +9644,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>0</v>
       </c>
@@ -9941,7 +9671,6 @@
       <c r="C13" t="n">
         <v>11144314.06999996</v>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -9969,7 +9698,6 @@
       <c r="C14" t="n">
         <v>32811735.26999999</v>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>105051</v>
       </c>
@@ -9997,7 +9725,6 @@
       <c r="C15" t="n">
         <v>32554696.85000001</v>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>406256</v>
       </c>
@@ -10025,7 +9752,6 @@
       <c r="C16" t="n">
         <v>16433170.41</v>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>103778</v>
       </c>
@@ -10050,8 +9776,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>0</v>
       </c>
@@ -10076,8 +9800,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
         <v>0</v>
       </c>
@@ -10105,7 +9827,6 @@
       <c r="C19" t="n">
         <v>11842891.11</v>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>0</v>
       </c>
@@ -10133,7 +9854,6 @@
       <c r="C20" t="n">
         <v>31785726.14</v>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>104606</v>
       </c>
@@ -10161,7 +9881,6 @@
       <c r="C21" t="n">
         <v>32494177.39000001</v>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>415715</v>
       </c>
@@ -10189,7 +9908,6 @@
       <c r="C22" t="n">
         <v>16534371.15</v>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>104939</v>
       </c>
@@ -10214,8 +9932,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>0</v>
       </c>
@@ -10240,8 +9956,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>0</v>
       </c>
@@ -10269,7 +9983,6 @@
       <c r="C25" t="n">
         <v>13148834.95</v>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -10297,7 +10010,6 @@
       <c r="C26" t="n">
         <v>31585702.67000001</v>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>104695</v>
       </c>
@@ -10325,7 +10037,6 @@
       <c r="C27" t="n">
         <v>32978250.01000001</v>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>408999</v>
       </c>
@@ -10353,7 +10064,6 @@
       <c r="C28" t="n">
         <v>16542746.73</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>105189</v>
       </c>
@@ -10378,8 +10088,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>0</v>
       </c>
@@ -10404,8 +10112,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>0</v>
       </c>
@@ -10433,7 +10139,6 @@
       <c r="C31" t="n">
         <v>12121275.75999999</v>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>0</v>
       </c>
@@ -10461,7 +10166,6 @@
       <c r="C32" t="n">
         <v>31706829.31999999</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>104853</v>
       </c>
@@ -10489,7 +10193,6 @@
       <c r="C33" t="n">
         <v>31780975.36000001</v>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>402155</v>
       </c>
@@ -10517,7 +10220,6 @@
       <c r="C34" t="n">
         <v>16380367.26</v>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>104516</v>
       </c>
@@ -10542,8 +10244,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0</v>
       </c>
@@ -10568,8 +10268,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>0</v>
       </c>
@@ -10597,7 +10295,6 @@
       <c r="C37" t="n">
         <v>11461000.25000001</v>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0</v>
       </c>
@@ -10625,7 +10322,6 @@
       <c r="C38" t="n">
         <v>31541938.83</v>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>105409</v>
       </c>
@@ -10653,7 +10349,6 @@
       <c r="C39" t="n">
         <v>33286091.14</v>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>405228</v>
       </c>
@@ -10681,7 +10376,6 @@
       <c r="C40" t="n">
         <v>16286342.84</v>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>105018</v>
       </c>
@@ -10706,8 +10400,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -10732,8 +10424,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -10761,7 +10451,6 @@
       <c r="C43" t="n">
         <v>10856595.95999999</v>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>0</v>
       </c>
@@ -10789,7 +10478,6 @@
       <c r="C44" t="n">
         <v>31695086.45</v>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>105592</v>
       </c>
@@ -10817,7 +10505,6 @@
       <c r="C45" t="n">
         <v>31523953.94</v>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>398400</v>
       </c>
@@ -10845,7 +10532,6 @@
       <c r="C46" t="n">
         <v>16495358.19</v>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>104708</v>
       </c>
@@ -10870,8 +10556,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>0</v>
       </c>
@@ -10896,8 +10580,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0</v>
       </c>
@@ -10925,7 +10607,6 @@
       <c r="C49" t="n">
         <v>10539179.13999999</v>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0</v>
       </c>
@@ -10953,7 +10634,6 @@
       <c r="C50" t="n">
         <v>31756830.82</v>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>107204</v>
       </c>
@@ -10981,7 +10661,6 @@
       <c r="C51" t="n">
         <v>33648299.87</v>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>407702</v>
       </c>
@@ -11009,7 +10688,6 @@
       <c r="C52" t="n">
         <v>16609379.18</v>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>105134</v>
       </c>
@@ -11034,8 +10712,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
         <v>0</v>
       </c>
@@ -11060,8 +10736,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>0</v>
       </c>
@@ -11089,7 +10763,6 @@
       <c r="C55" t="n">
         <v>11524594.71999997</v>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0</v>
       </c>
@@ -11117,7 +10790,6 @@
       <c r="C56" t="n">
         <v>31924428.03999999</v>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>107374</v>
       </c>
@@ -11145,7 +10817,6 @@
       <c r="C57" t="n">
         <v>31947440.25</v>
       </c>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>401325</v>
       </c>
@@ -11173,7 +10844,6 @@
       <c r="C58" t="n">
         <v>16450194.76</v>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>103936</v>
       </c>
@@ -11198,8 +10868,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>0</v>
       </c>
@@ -11224,8 +10892,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>0</v>
       </c>
@@ -11253,7 +10919,6 @@
       <c r="C61" t="n">
         <v>10554548.78000002</v>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>0</v>
       </c>
@@ -11281,7 +10946,6 @@
       <c r="C62" t="n">
         <v>32012386.53000001</v>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>106525</v>
       </c>
@@ -11309,7 +10973,6 @@
       <c r="C63" t="n">
         <v>30407306.1</v>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>393549</v>
       </c>
@@ -11337,7 +11000,6 @@
       <c r="C64" t="n">
         <v>15773882.06</v>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>102974</v>
       </c>
@@ -11362,8 +11024,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0</v>
       </c>
@@ -11388,8 +11048,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>0</v>
       </c>
@@ -11417,7 +11075,6 @@
       <c r="C67" t="n">
         <v>9831177.919999987</v>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>0</v>
       </c>
@@ -11445,7 +11102,6 @@
       <c r="C68" t="n">
         <v>31420732.48</v>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>106046</v>
       </c>
@@ -11473,7 +11129,6 @@
       <c r="C69" t="n">
         <v>32036128.32</v>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>399776</v>
       </c>
@@ -11501,7 +11156,6 @@
       <c r="C70" t="n">
         <v>16247699.7</v>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>102423</v>
       </c>
@@ -11526,8 +11180,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>0</v>
       </c>
@@ -11552,8 +11204,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>0</v>
       </c>
@@ -11581,7 +11231,6 @@
       <c r="C73" t="n">
         <v>35568610.43000001</v>
       </c>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>0</v>
       </c>
@@ -11696,8 +11345,6 @@
           <t>TV</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>0</v>
       </c>
@@ -11722,8 +11369,6 @@
           <t>Residential Security</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>0</v>
       </c>
@@ -11751,7 +11396,6 @@
       <c r="C79" t="n">
         <v>27401112.98000621</v>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>0</v>
       </c>
@@ -11778,6 +11422,17 @@
   </sheetPr>
   <dimension ref="A1:I105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="13.85546875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="12" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14.7109375" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="12.28515625" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="5.140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="12" bestFit="1" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -11840,7 +11495,6 @@
       <c r="C2" t="n">
         <v>12623062.6</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
         <v>0</v>
       </c>
@@ -11871,7 +11525,6 @@
       <c r="C3" t="n">
         <v>2588219.58</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
         <v>0</v>
       </c>
@@ -11902,7 +11555,6 @@
       <c r="C4" t="n">
         <v>4344979.85</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -11933,7 +11585,6 @@
       <c r="C5" t="n">
         <v>21111329.68</v>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -11964,7 +11615,6 @@
       <c r="C6" t="n">
         <v>3736200.02</v>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>0</v>
       </c>
@@ -11995,7 +11645,6 @@
       <c r="C7" t="n">
         <v>489552.09</v>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>0</v>
       </c>
@@ -12026,7 +11675,6 @@
       <c r="C8" t="n">
         <v>-2388946.55</v>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>0</v>
       </c>
@@ -12054,8 +11702,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>0</v>
       </c>
@@ -12086,7 +11732,6 @@
       <c r="C10" t="n">
         <v>13278641.04</v>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
         <v>0</v>
       </c>
@@ -12117,7 +11762,6 @@
       <c r="C11" t="n">
         <v>2763986.64</v>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
         <v>0</v>
       </c>
@@ -12148,7 +11792,6 @@
       <c r="C12" t="n">
         <v>3902053.16</v>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>0</v>
       </c>
@@ -12179,7 +11822,6 @@
       <c r="C13" t="n">
         <v>23020111.6</v>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
         <v>0</v>
       </c>
@@ -12210,7 +11852,6 @@
       <c r="C14" t="n">
         <v>3860684.96</v>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
         <v>0</v>
       </c>
@@ -12241,7 +11882,6 @@
       <c r="C15" t="n">
         <v>496473.19</v>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="n">
         <v>0</v>
       </c>
@@ -12272,7 +11912,6 @@
       <c r="C16" t="n">
         <v>70522.28999999954</v>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="n">
         <v>0</v>
       </c>
@@ -12300,8 +11939,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
         <v>0</v>
       </c>
@@ -12332,7 +11969,6 @@
       <c r="C18" t="n">
         <v>12914340.37</v>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
         <v>0</v>
       </c>
@@ -12363,7 +11999,6 @@
       <c r="C19" t="n">
         <v>2739404.110000001</v>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
         <v>0</v>
       </c>
@@ -12394,7 +12029,6 @@
       <c r="C20" t="n">
         <v>3879872.13</v>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
         <v>0</v>
       </c>
@@ -12425,7 +12059,6 @@
       <c r="C21" t="n">
         <v>24194644.12</v>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>0</v>
       </c>
@@ -12456,7 +12089,6 @@
       <c r="C22" t="n">
         <v>3725848.62</v>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="n">
         <v>0</v>
       </c>
@@ -12487,7 +12119,6 @@
       <c r="C23" t="n">
         <v>478223.72</v>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
         <v>0</v>
       </c>
@@ -12518,7 +12149,6 @@
       <c r="C24" t="n">
         <v>-2171392.180000005</v>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>0</v>
       </c>
@@ -12546,8 +12176,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>0</v>
       </c>
@@ -12578,7 +12206,6 @@
       <c r="C26" t="n">
         <v>13265097.9</v>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>0</v>
       </c>
@@ -12609,7 +12236,6 @@
       <c r="C27" t="n">
         <v>2743690.700000001</v>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>0</v>
       </c>
@@ -12640,7 +12266,6 @@
       <c r="C28" t="n">
         <v>3495626.21</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
         <v>0</v>
       </c>
@@ -12671,7 +12296,6 @@
       <c r="C29" t="n">
         <v>22292104.04</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
         <v>0</v>
       </c>
@@ -12702,7 +12326,6 @@
       <c r="C30" t="n">
         <v>3865294.77</v>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
         <v>0</v>
       </c>
@@ -12733,7 +12356,6 @@
       <c r="C31" t="n">
         <v>492742.61</v>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>0</v>
       </c>
@@ -12764,7 +12386,6 @@
       <c r="C32" t="n">
         <v>-25886.27000000088</v>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>0</v>
       </c>
@@ -12792,8 +12413,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>0</v>
       </c>
@@ -12824,7 +12443,6 @@
       <c r="C34" t="n">
         <v>13365167.1</v>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
         <v>0</v>
       </c>
@@ -12855,7 +12473,6 @@
       <c r="C35" t="n">
         <v>2727053.620000001</v>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
         <v>0</v>
       </c>
@@ -12886,7 +12503,6 @@
       <c r="C36" t="n">
         <v>3524553.02</v>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>0</v>
       </c>
@@ -12917,7 +12533,6 @@
       <c r="C37" t="n">
         <v>23951841.04</v>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0</v>
       </c>
@@ -12948,7 +12563,6 @@
       <c r="C38" t="n">
         <v>3618244.21</v>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>0</v>
       </c>
@@ -12979,7 +12593,6 @@
       <c r="C39" t="n">
         <v>469204.1299999999</v>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="n">
         <v>0</v>
       </c>
@@ -13010,7 +12623,6 @@
       <c r="C40" t="n">
         <v>436868.220000008</v>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
         <v>0</v>
       </c>
@@ -13038,8 +12650,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -13070,7 +12680,6 @@
       <c r="C42" t="n">
         <v>13015129.58</v>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -13101,7 +12710,6 @@
       <c r="C43" t="n">
         <v>2704582.71</v>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>0</v>
       </c>
@@ -13132,7 +12740,6 @@
       <c r="C44" t="n">
         <v>3389763.510000001</v>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>0</v>
       </c>
@@ -13163,7 +12770,6 @@
       <c r="C45" t="n">
         <v>24837872.53</v>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>0</v>
       </c>
@@ -13194,7 +12800,6 @@
       <c r="C46" t="n">
         <v>3744977.33</v>
       </c>
-      <c r="D46" t="inlineStr"/>
       <c r="E46" t="n">
         <v>0</v>
       </c>
@@ -13225,7 +12830,6 @@
       <c r="C47" t="n">
         <v>470858.03</v>
       </c>
-      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>0</v>
       </c>
@@ -13256,7 +12860,6 @@
       <c r="C48" t="n">
         <v>717630.6599999904</v>
       </c>
-      <c r="D48" t="inlineStr"/>
       <c r="E48" t="n">
         <v>0</v>
       </c>
@@ -13284,8 +12887,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="n">
         <v>0</v>
       </c>
@@ -13316,7 +12917,6 @@
       <c r="C50" t="n">
         <v>12857507.04</v>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="n">
         <v>0</v>
       </c>
@@ -13347,7 +12947,6 @@
       <c r="C51" t="n">
         <v>2737258.27</v>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>0</v>
       </c>
@@ -13378,7 +12977,6 @@
       <c r="C52" t="n">
         <v>3344374.77</v>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>0</v>
       </c>
@@ -13409,7 +13007,6 @@
       <c r="C53" t="n">
         <v>24657798.08000001</v>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
         <v>0</v>
       </c>
@@ -13440,7 +13037,6 @@
       <c r="C54" t="n">
         <v>3752634.69</v>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
         <v>0</v>
       </c>
@@ -13471,7 +13067,6 @@
       <c r="C55" t="n">
         <v>470973.66</v>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>0</v>
       </c>
@@ -13502,7 +13097,6 @@
       <c r="C56" t="n">
         <v>-1799860.500000008</v>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="n">
         <v>0</v>
       </c>
@@ -13530,8 +13124,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>0</v>
       </c>
@@ -13562,7 +13154,6 @@
       <c r="C58" t="n">
         <v>13235260.51</v>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>0</v>
       </c>
@@ -13593,7 +13184,6 @@
       <c r="C59" t="n">
         <v>2794737.33</v>
       </c>
-      <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
         <v>0</v>
       </c>
@@ -13624,7 +13214,6 @@
       <c r="C60" t="n">
         <v>3419255.28</v>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="n">
         <v>0</v>
       </c>
@@ -13655,7 +13244,6 @@
       <c r="C61" t="n">
         <v>23633700.19</v>
       </c>
-      <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
         <v>0</v>
       </c>
@@ -13686,7 +13274,6 @@
       <c r="C62" t="n">
         <v>3749461.86</v>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>0</v>
       </c>
@@ -13717,7 +13304,6 @@
       <c r="C63" t="n">
         <v>461242.88</v>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>0</v>
       </c>
@@ -13748,7 +13334,6 @@
       <c r="C64" t="n">
         <v>-2180681.550000003</v>
       </c>
-      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>0</v>
       </c>
@@ -13776,8 +13361,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0</v>
       </c>
@@ -13808,7 +13391,6 @@
       <c r="C66" t="n">
         <v>13124633.87</v>
       </c>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="n">
         <v>0</v>
       </c>
@@ -13839,7 +13421,6 @@
       <c r="C67" t="n">
         <v>3249438.47</v>
       </c>
-      <c r="D67" t="inlineStr"/>
       <c r="E67" t="n">
         <v>0</v>
       </c>
@@ -13870,7 +13451,6 @@
       <c r="C68" t="n">
         <v>3443355.58</v>
       </c>
-      <c r="D68" t="inlineStr"/>
       <c r="E68" t="n">
         <v>0</v>
       </c>
@@ -13901,7 +13481,6 @@
       <c r="C69" t="n">
         <v>27059563.28</v>
       </c>
-      <c r="D69" t="inlineStr"/>
       <c r="E69" t="n">
         <v>0</v>
       </c>
@@ -13932,7 +13511,6 @@
       <c r="C70" t="n">
         <v>3848071.37</v>
       </c>
-      <c r="D70" t="inlineStr"/>
       <c r="E70" t="n">
         <v>0</v>
       </c>
@@ -13963,7 +13541,6 @@
       <c r="C71" t="n">
         <v>465963.25</v>
       </c>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>0</v>
       </c>
@@ -13994,7 +13571,6 @@
       <c r="C72" t="n">
         <v>-2501556.88000001</v>
       </c>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>0</v>
       </c>
@@ -14022,8 +13598,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>0</v>
       </c>
@@ -14054,7 +13628,6 @@
       <c r="C74" t="n">
         <v>12869614.99</v>
       </c>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" t="n">
         <v>0</v>
       </c>
@@ -14085,7 +13658,6 @@
       <c r="C75" t="n">
         <v>2987306.63</v>
       </c>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
         <v>0</v>
       </c>
@@ -14116,7 +13688,6 @@
       <c r="C76" t="n">
         <v>4003784.07</v>
       </c>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>0</v>
       </c>
@@ -14147,7 +13718,6 @@
       <c r="C77" t="n">
         <v>21777020.56</v>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>0</v>
       </c>
@@ -14178,7 +13748,6 @@
       <c r="C78" t="n">
         <v>3749043.75</v>
       </c>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>0</v>
       </c>
@@ -14209,7 +13778,6 @@
       <c r="C79" t="n">
         <v>458438.66</v>
       </c>
-      <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>0</v>
       </c>
@@ -14240,7 +13808,6 @@
       <c r="C80" t="n">
         <v>-1754001.680000002</v>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
         <v>0</v>
       </c>
@@ -14268,8 +13835,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr"/>
-      <c r="D81" t="inlineStr"/>
       <c r="E81" t="n">
         <v>0</v>
       </c>
@@ -14300,7 +13865,6 @@
       <c r="C82" t="n">
         <v>12306095.63</v>
       </c>
-      <c r="D82" t="inlineStr"/>
       <c r="E82" t="n">
         <v>0</v>
       </c>
@@ -14331,7 +13895,6 @@
       <c r="C83" t="n">
         <v>2906828.77</v>
       </c>
-      <c r="D83" t="inlineStr"/>
       <c r="E83" t="n">
         <v>0</v>
       </c>
@@ -14362,7 +13925,6 @@
       <c r="C84" t="n">
         <v>2756960.31</v>
       </c>
-      <c r="D84" t="inlineStr"/>
       <c r="E84" t="n">
         <v>0</v>
       </c>
@@ -14393,7 +13955,6 @@
       <c r="C85" t="n">
         <v>26517657.66</v>
       </c>
-      <c r="D85" t="inlineStr"/>
       <c r="E85" t="n">
         <v>0</v>
       </c>
@@ -14424,7 +13985,6 @@
       <c r="C86" t="n">
         <v>3450194.39</v>
       </c>
-      <c r="D86" t="inlineStr"/>
       <c r="E86" t="n">
         <v>0</v>
       </c>
@@ -14455,7 +14015,6 @@
       <c r="C87" t="n">
         <v>453998.5599999999</v>
       </c>
-      <c r="D87" t="inlineStr"/>
       <c r="E87" t="n">
         <v>0</v>
       </c>
@@ -14486,7 +14045,6 @@
       <c r="C88" t="n">
         <v>-1027449.279999999</v>
       </c>
-      <c r="D88" t="inlineStr"/>
       <c r="E88" t="n">
         <v>0</v>
       </c>
@@ -14514,8 +14072,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
       <c r="E89" t="n">
         <v>0</v>
       </c>
@@ -14546,7 +14102,6 @@
       <c r="C90" t="n">
         <v>13562074.76</v>
       </c>
-      <c r="D90" t="inlineStr"/>
       <c r="E90" t="n">
         <v>0</v>
       </c>
@@ -14577,7 +14132,6 @@
       <c r="C91" t="n">
         <v>3190898.120000001</v>
       </c>
-      <c r="D91" t="inlineStr"/>
       <c r="E91" t="n">
         <v>0</v>
       </c>
@@ -14608,7 +14162,6 @@
       <c r="C92" t="n">
         <v>3488349.079999999</v>
       </c>
-      <c r="D92" t="inlineStr"/>
       <c r="E92" t="n">
         <v>0</v>
       </c>
@@ -14639,7 +14192,6 @@
       <c r="C93" t="n">
         <v>23310994.27</v>
       </c>
-      <c r="D93" t="inlineStr"/>
       <c r="E93" t="n">
         <v>0</v>
       </c>
@@ -14670,7 +14222,6 @@
       <c r="C94" t="n">
         <v>3837644.59</v>
       </c>
-      <c r="D94" t="inlineStr"/>
       <c r="E94" t="n">
         <v>0</v>
       </c>
@@ -14701,7 +14252,6 @@
       <c r="C95" t="n">
         <v>429191.72</v>
       </c>
-      <c r="D95" t="inlineStr"/>
       <c r="E95" t="n">
         <v>0</v>
       </c>
@@ -14732,7 +14282,6 @@
       <c r="C96" t="n">
         <v>29994897.77000001</v>
       </c>
-      <c r="D96" t="inlineStr"/>
       <c r="E96" t="n">
         <v>0</v>
       </c>
@@ -14760,8 +14309,6 @@
           <t>IoT</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr"/>
-      <c r="D97" t="inlineStr"/>
       <c r="E97" t="n">
         <v>0</v>
       </c>

</xml_diff>